<commit_message>
docs: add product catalogue test scenarios and test cases
</commit_message>
<xml_diff>
--- a/test-cases/SauceDemo_TestCases.xlsx
+++ b/test-cases/SauceDemo_TestCases.xlsx
@@ -1,17 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\saucedemo-playwright-pom\test-cases\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88E1F1F0-E795-4C50-8453-7727C97E32E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Login" sheetId="1" r:id="rId5"/>
+    <sheet name="Login" sheetId="1" r:id="rId1"/>
+    <sheet name="Product Catalogue" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="200">
   <si>
     <t>Field</t>
   </si>
@@ -63,20 +73,19 @@
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
         <rFont val="Times"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="12.0"/>
       </rPr>
       <t xml:space="preserve">Common Login Preconditions :
 </t>
     </r>
     <r>
       <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
         <rFont val="Times"/>
-        <b val="0"/>
-        <color theme="1"/>
-        <sz val="12.0"/>
       </rPr>
       <t xml:space="preserve">Sauce Demo application is accessible.        
 User is on the Login page.        
@@ -86,20 +95,19 @@
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
         <rFont val="Times"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="12.0"/>
       </rPr>
       <t xml:space="preserve">Common Test Steps :
 </t>
     </r>
     <r>
       <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
         <rFont val="Times"/>
-        <b val="0"/>
-        <color theme="1"/>
-        <sz val="12.0"/>
       </rPr>
       <t>1. Launch the Sauce Demo application.
 2. Enter the username as specified in the test data.
@@ -292,41 +300,556 @@
 2. User should not be logged in.
 3. User should remain on the Login page.</t>
   </si>
+  <si>
+    <t>Product Catalogue</t>
+  </si>
+  <si>
+    <t>TS_PRODUCT_001</t>
+  </si>
+  <si>
+    <t>Verify the layout and UI elements of the Product Listing page </t>
+  </si>
+  <si>
+    <t>TS_PRODUCT_002</t>
+  </si>
+  <si>
+    <t>Verify product details displayed on the Product Listing page </t>
+  </si>
+  <si>
+    <t>TS_PRODUCT_003</t>
+  </si>
+  <si>
+    <t>Verify product sorting functionality based on available sorting options </t>
+  </si>
+  <si>
+    <t>TS_PRODUCT_004</t>
+  </si>
+  <si>
+    <t>Verify navigation to the Product Details page from Product Listing page </t>
+  </si>
+  <si>
+    <t>TS_PRODUCT_005</t>
+  </si>
+  <si>
+    <t>Verify user can add single and multiple products to the shopping cart </t>
+  </si>
+  <si>
+    <t>TS_PRODUCT_006</t>
+  </si>
+  <si>
+    <t>Verify user can remove single and multiple products from the shopping cart </t>
+  </si>
+  <si>
+    <t>TS_PRODUCT_007</t>
+  </si>
+  <si>
+    <t>Verify navigation from Product Listing page to Shopping Cart page </t>
+  </si>
+  <si>
+    <t>TS_PRODUCT_008</t>
+  </si>
+  <si>
+    <t>Verify added products persist in the cart until they are removed </t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_001</t>
+  </si>
+  <si>
+    <t>Verify the title of the Product Listing page</t>
+  </si>
+  <si>
+    <t>Common Product Catalogue Preconditions</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>1. Verify the page title.</t>
+  </si>
+  <si>
+    <t>Page title should be displayed correctly as "Products".</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_002</t>
+  </si>
+  <si>
+    <t>Verify menu button and cart icon are displayed on the Product Listing page</t>
+  </si>
+  <si>
+    <t>1. Verify the menu button. 
+2. Verify the cart icon.</t>
+  </si>
+  <si>
+    <t>Menu button and cart icon should be displayed and visible on the Product Listing page.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_003</t>
+  </si>
+  <si>
+    <t>Verify product inventory section is displayed on the Product Listing page</t>
+  </si>
+  <si>
+    <t>1. Verify the product inventory section.</t>
+  </si>
+  <si>
+    <t>Product inventory section containing available products should be displayed.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_004</t>
+  </si>
+  <si>
+    <t>Verify each product card displays product image, name, description, and price</t>
+  </si>
+  <si>
+    <t>Available products</t>
+  </si>
+  <si>
+    <t>1. Verify each product card. 
+2. Verify the product image. 
+3. Verify the product name. 
+4. Verify the product description. 
+5. Verify the product price.</t>
+  </si>
+  <si>
+    <t>Each product card should display a product image, name, description, and price.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_005</t>
+  </si>
+  <si>
+    <t>Verify all product names are unique</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Product names from inventory</t>
+  </si>
+  <si>
+    <t>1. Capture all product names. 
+2. Compare the product names for duplicates.</t>
+  </si>
+  <si>
+    <t>All product names displayed should be unique.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_006</t>
+  </si>
+  <si>
+    <t>Verify all product prices are greater than zero</t>
+  </si>
+  <si>
+    <t>Product prices</t>
+  </si>
+  <si>
+    <t>1. Capture all product prices. 
+2. Remove the currency symbol from each price. 
+3. Verify that each price is greater than zero.</t>
+  </si>
+  <si>
+    <t>All displayed product prices should be greater than zero.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_007</t>
+  </si>
+  <si>
+    <t>Verify product images are displayed and loaded successfully</t>
+  </si>
+  <si>
+    <t>Product images</t>
+  </si>
+  <si>
+    <t>1. Verify each product image is visible. 
+2. Verify each product image has a valid image source.</t>
+  </si>
+  <si>
+    <t>Product images should be displayed and loaded successfully for all products.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_008</t>
+  </si>
+  <si>
+    <t>Verify products are sorted by Name (A-Z) by default</t>
+  </si>
+  <si>
+    <t>Default sorting: Name (A-Z)</t>
+  </si>
+  <si>
+    <t>1. Capture the displayed product names. 
+2. Compare the product names with ascending alphabetical order. 
+3. Verify the selected sorting option.</t>
+  </si>
+  <si>
+    <t>Products should be displayed in ascending alphabetical order by default, and Name (A-Z) should be selected.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_009</t>
+  </si>
+  <si>
+    <t>Verify product sorting by Name (Z-A)</t>
+  </si>
+  <si>
+    <t>Sort option: Name (Z-A)</t>
+  </si>
+  <si>
+    <t>1. Select Name (Z-A) from the sorting dropdown. 
+2. Capture the displayed product names. 
+3. Compare the product names with descending alphabetical order.</t>
+  </si>
+  <si>
+    <t>Products should be sorted alphabetically from Z to A.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_010</t>
+  </si>
+  <si>
+    <t>Verify product sorting by Price (Low to High)</t>
+  </si>
+  <si>
+    <t>Sort option: Price (Low to High)</t>
+  </si>
+  <si>
+    <t>1. Select Price (Low to High) from the sorting dropdown. 
+2. Capture the displayed product prices. 
+3. Compare the prices with ascending numerical order.</t>
+  </si>
+  <si>
+    <t>Products should be sorted from the lowest price to the highest price.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_011</t>
+  </si>
+  <si>
+    <t>Verify product sorting by Price (High to Low)</t>
+  </si>
+  <si>
+    <t>Sort option: Price (High to Low)</t>
+  </si>
+  <si>
+    <t>1. Select Price (High to Low) from the sorting dropdown. 
+2. Capture the displayed product prices. 
+3. Compare the prices with descending numerical order.</t>
+  </si>
+  <si>
+    <t>Products should be sorted from the highest price to the lowest price.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_012</t>
+  </si>
+  <si>
+    <t>Verify selected sorting option is displayed correctly after applying sorting</t>
+  </si>
+  <si>
+    <t>Available sorting options</t>
+  </si>
+  <si>
+    <t>1. Select a sorting option. 
+2. Verify the selected value in the sorting dropdown.</t>
+  </si>
+  <si>
+    <t>The selected sorting option should be displayed correctly in the sorting dropdown.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_013</t>
+  </si>
+  <si>
+    <t>Verify sorting works correctly after adding a product to the cart</t>
+  </si>
+  <si>
+    <t>Product: Sauce Labs Backpack</t>
+  </si>
+  <si>
+    <t>1. Add the selected product to the cart. 
+2. Select a sorting option. 
+3. Verify the product ordering.</t>
+  </si>
+  <si>
+    <t>Sorting functionality should work correctly after adding a product to the cart.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_014</t>
+  </si>
+  <si>
+    <t>Verify sorting does not affect the cart badge count</t>
+  </si>
+  <si>
+    <t>1. Note the cart badge count. 
+2. Apply different sorting options. 
+3. Verify the cart badge count.</t>
+  </si>
+  <si>
+    <t>Sorting products should not change the cart badge count.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_015</t>
+  </si>
+  <si>
+    <t>Verify clicking a product name navigates to the Product Details page</t>
+  </si>
+  <si>
+    <t>1. Click the product name. 
+2. Verify navigation to the Product Details page.</t>
+  </si>
+  <si>
+    <t>User should be navigated to the Product Details page of the selected product.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_016</t>
+  </si>
+  <si>
+    <t>Verify product details match the selected product</t>
+  </si>
+  <si>
+    <t>1. Capture the selected product's name, image, description, and price. 
+2. Open the Product Details page for the selected product. 
+3. Compare the product details.</t>
+  </si>
+  <si>
+    <t>Product Details page should display the same product name, image, description, and price as the selected product.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_017</t>
+  </si>
+  <si>
+    <t>Verify user is redirected to the Cart page by clicking the cart icon</t>
+  </si>
+  <si>
+    <t>1. Click the cart icon. 
+2. Verify navigation to the Cart page.</t>
+  </si>
+  <si>
+    <t>User should be redirected successfully to the Cart page.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_018</t>
+  </si>
+  <si>
+    <t>Verify user can add a single product to the cart</t>
+  </si>
+  <si>
+    <t>1. Click Add to Cart for the selected product. 
+2. Verify the cart badge count. 
+3. Open the Cart page. 
+4. Verify the selected product.</t>
+  </si>
+  <si>
+    <t>Selected product should be added successfully to the cart. 
+Cart badge should display 1, and the selected product should be displayed in the cart.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_019</t>
+  </si>
+  <si>
+    <t>Verify user can add multiple products to the cart</t>
+  </si>
+  <si>
+    <t>1. Click Add to Cart for the first product. 
+2. Click Add to Cart for the second product. 
+3. Verify the cart badge count. 
+4. Open the Cart page. 
+5. Verify the selected products.</t>
+  </si>
+  <si>
+    <t>All selected products should be added successfully. 
+Cart badge should display the total number of products added, and all selected products should be displayed in the cart.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_020</t>
+  </si>
+  <si>
+    <t>Verify user can remove a single product from the cart</t>
+  </si>
+  <si>
+    <t>Common Product Catalogue Preconditions;
+Selected product is already present in the cart</t>
+  </si>
+  <si>
+    <t>1. Open the Cart page. 
+2. Note the current cart badge count. 
+3. Click Remove for the selected product. 
+4. Verify the product is no longer displayed. 
+5. Verify the cart badge count.</t>
+  </si>
+  <si>
+    <t>Selected product should be removed successfully, and the cart badge count should decrease by 1.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_021</t>
+  </si>
+  <si>
+    <t>Verify user can remove multiple products from the cart</t>
+  </si>
+  <si>
+    <t>Common Product Catalogue Preconditions;
+Multiple products are already present in the cart</t>
+  </si>
+  <si>
+    <t>1. Open the Cart page. 
+2. Note the current cart badge count. 
+3. Click Remove for each selected product. 
+4. Verify the selected products are no longer displayed. 
+5. Verify the cart badge count.</t>
+  </si>
+  <si>
+    <t>All selected products should be removed successfully, and the cart badge count should decrease according to the number of products removed.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_022</t>
+  </si>
+  <si>
+    <t>Verify added products persist after refreshing the page</t>
+  </si>
+  <si>
+    <t>1. Refresh the Product Listing page. 
+2. Open the Cart page. 
+3. Verify the selected product.</t>
+  </si>
+  <si>
+    <t>The added product should remain in the cart after the page is refreshed.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_023</t>
+  </si>
+  <si>
+    <t>Verify added products persist when navigating between Product Listing and Cart pages</t>
+  </si>
+  <si>
+    <t>1. Navigate to the Cart page. 
+2. Navigate back to the Product Listing page. 
+3. Navigate to the Cart page again. 
+4. Verify the selected product.</t>
+  </si>
+  <si>
+    <t>The added product should remain in the cart while navigating between the Product Listing and Cart pages.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Common Product Catalogue Preconditions :
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>1. Sauce Demo application is accessible.
+2. User is logged in successfully.
+3. Product Listing page is displayed.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">Common Test Steps :
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>1. Launch the Sauce Demo application.
+2. Enter the username.
+3. Enter the password.
+4. Click the Login button.</t>
+    </r>
+  </si>
+  <si>
+    <t>Product: Sauce Labs Fleece Jacket</t>
+  </si>
+  <si>
+    <t>Products: Backpack + Bike Light + Fleece Jacket (3 products)</t>
+  </si>
+  <si>
+    <t>Product: Backpack + Bike Light + Fleece Jacket (3 products)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Times"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Times"/>
     </font>
-    <font/>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -334,9 +857,21 @@
         <bgColor rgb="FFCCCCCC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCCCCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
-    <border/>
+  <borders count="5">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
@@ -350,19 +885,23 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
+      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
@@ -372,67 +911,108 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="25">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -622,27 +1202,30 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:H27"/>
+  <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="18.5"/>
-    <col customWidth="1" min="2" max="2" width="25.13"/>
-    <col customWidth="1" min="3" max="3" width="42.75"/>
-    <col customWidth="1" min="4" max="4" width="7.75"/>
-    <col customWidth="1" min="5" max="5" width="25.25"/>
-    <col customWidth="1" min="6" max="6" width="30.13"/>
-    <col customWidth="1" min="7" max="7" width="17.13"/>
-    <col customWidth="1" min="8" max="8" width="65.13"/>
+    <col min="1" max="1" width="18.46484375" customWidth="1"/>
+    <col min="2" max="2" width="25.1328125" customWidth="1"/>
+    <col min="3" max="3" width="42.73046875" customWidth="1"/>
+    <col min="4" max="4" width="7.73046875" customWidth="1"/>
+    <col min="5" max="5" width="25.265625" customWidth="1"/>
+    <col min="6" max="6" width="30.1328125" customWidth="1"/>
+    <col min="7" max="7" width="17.1328125" customWidth="1"/>
+    <col min="8" max="8" width="65.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -656,7 +1239,7 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
     </row>
-    <row r="2">
+    <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
@@ -670,7 +1253,7 @@
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
     </row>
-    <row r="3">
+    <row r="3" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -684,7 +1267,7 @@
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
     </row>
-    <row r="4">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -694,77 +1277,77 @@
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
     </row>
-    <row r="5">
+    <row r="5" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="7"/>
+      <c r="C5" s="10"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
     </row>
-    <row r="6">
-      <c r="A6" s="8" t="s">
+    <row r="6" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="7"/>
+      <c r="C6" s="10"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
     </row>
-    <row r="7">
-      <c r="A7" s="8" t="s">
+    <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="7"/>
+      <c r="C7" s="10"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
     </row>
-    <row r="8">
-      <c r="A8" s="8" t="s">
+    <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A8" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="7"/>
+      <c r="C8" s="10"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
     </row>
-    <row r="9">
-      <c r="A9" s="8" t="s">
+    <row r="9" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A9" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="7"/>
+      <c r="C9" s="10"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
     </row>
-    <row r="10">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -774,11 +1357,11 @@
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
     </row>
-    <row r="11">
-      <c r="A11" s="10" t="s">
+    <row r="11" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A11" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="7"/>
+      <c r="B11" s="10"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
@@ -786,7 +1369,7 @@
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
     </row>
-    <row r="12">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -796,11 +1379,11 @@
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
     </row>
-    <row r="13">
-      <c r="A13" s="10" t="s">
+    <row r="13" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A13" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="7"/>
+      <c r="B13" s="10"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
@@ -808,7 +1391,7 @@
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
     </row>
-    <row r="14">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -818,33 +1401,33 @@
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
     </row>
-    <row r="15">
-      <c r="A15" s="11" t="s">
+    <row r="15" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="D15" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="E15" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="F15" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G15" s="11" t="s">
+      <c r="G15" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="H15" s="11" t="s">
+      <c r="H15" s="7" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="3" t="s">
         <v>26</v>
       </c>
@@ -870,7 +1453,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="3" t="s">
         <v>33</v>
       </c>
@@ -896,7 +1479,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="3" t="s">
         <v>37</v>
       </c>
@@ -922,7 +1505,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="3" t="s">
         <v>40</v>
       </c>
@@ -948,7 +1531,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="3" t="s">
         <v>43</v>
       </c>
@@ -974,14 +1557,14 @@
         <v>32</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="3" t="s">
         <v>46</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C21" s="12" t="s">
+      <c r="C21" s="8" t="s">
         <v>47</v>
       </c>
       <c r="D21" s="3" t="s">
@@ -1000,7 +1583,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="3" t="s">
         <v>50</v>
       </c>
@@ -1026,7 +1609,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="3" t="s">
         <v>53</v>
       </c>
@@ -1052,7 +1635,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A24" s="3" t="s">
         <v>56</v>
       </c>
@@ -1078,7 +1661,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A25" s="3" t="s">
         <v>60</v>
       </c>
@@ -1104,7 +1687,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A26" s="3" t="s">
         <v>64</v>
       </c>
@@ -1130,7 +1713,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A27" s="3" t="s">
         <v>67</v>
       </c>
@@ -1166,6 +1749,821 @@
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B9:C9"/>
   </mergeCells>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{791AF090-76B8-47F5-A4CB-9D7FC68A4A31}">
+  <dimension ref="A1:H42"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="22.06640625" customWidth="1"/>
+    <col min="2" max="2" width="22.59765625" customWidth="1"/>
+    <col min="3" max="3" width="71.46484375" customWidth="1"/>
+    <col min="4" max="4" width="7.9296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="37.06640625" customWidth="1"/>
+    <col min="6" max="6" width="31.06640625" customWidth="1"/>
+    <col min="7" max="7" width="61.59765625" customWidth="1"/>
+    <col min="8" max="8" width="68.3984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="15" x14ac:dyDescent="0.4">
+      <c r="A1" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="17" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A2" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A3" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="15" x14ac:dyDescent="0.35">
+      <c r="A5" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+    </row>
+    <row r="6" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+    </row>
+    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+    </row>
+    <row r="8" spans="1:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+    </row>
+    <row r="9" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+    </row>
+    <row r="10" spans="1:8" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+    </row>
+    <row r="11" spans="1:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+    </row>
+    <row r="12" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="C12" s="16"/>
+      <c r="D12" s="16"/>
+    </row>
+    <row r="13" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+    </row>
+    <row r="15" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A15" s="21" t="s">
+        <v>195</v>
+      </c>
+      <c r="B15" s="10"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="20"/>
+      <c r="G15" s="20"/>
+      <c r="H15" s="20"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A16" s="20"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="20"/>
+    </row>
+    <row r="17" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A17" s="22" t="s">
+        <v>196</v>
+      </c>
+      <c r="B17" s="23"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="20"/>
+      <c r="G17" s="20"/>
+      <c r="H17" s="20"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A18" s="20"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="20"/>
+      <c r="F18" s="20"/>
+      <c r="G18" s="20"/>
+      <c r="H18" s="20"/>
+    </row>
+    <row r="19" spans="1:8" ht="15" x14ac:dyDescent="0.4">
+      <c r="A19" s="24" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="C19" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="E19" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="F19" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="G19" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="H19" s="24" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
+      <c r="A20" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="B20" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="C20" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="D20" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E20" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="F20" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="G20" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="H20" s="18" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
+      <c r="A21" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="C21" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="D21" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E21" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="F21" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="G21" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="H21" s="18" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A22" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="D22" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="E22" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="F22" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="G22" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="H22" s="18" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A23" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="B23" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="C23" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="D23" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E23" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="F23" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="G23" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="H23" s="18" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
+      <c r="A24" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="B24" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="C24" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="D24" s="18" t="s">
+        <v>109</v>
+      </c>
+      <c r="E24" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="F24" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="G24" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="H24" s="18" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="46.15" x14ac:dyDescent="0.45">
+      <c r="A25" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="B25" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="D25" s="18" t="s">
+        <v>109</v>
+      </c>
+      <c r="E25" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="F25" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="G25" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="H25" s="18" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
+      <c r="A26" s="18" t="s">
+        <v>118</v>
+      </c>
+      <c r="B26" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="C26" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="D26" s="18" t="s">
+        <v>109</v>
+      </c>
+      <c r="E26" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="F26" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="G26" s="18" t="s">
+        <v>121</v>
+      </c>
+      <c r="H26" s="18" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="46.15" x14ac:dyDescent="0.45">
+      <c r="A27" s="18" t="s">
+        <v>123</v>
+      </c>
+      <c r="B27" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="C27" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="D27" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E27" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="F27" s="18" t="s">
+        <v>125</v>
+      </c>
+      <c r="G27" s="18" t="s">
+        <v>126</v>
+      </c>
+      <c r="H27" s="18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="46.15" x14ac:dyDescent="0.45">
+      <c r="A28" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="B28" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="C28" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="D28" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E28" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="F28" s="18" t="s">
+        <v>130</v>
+      </c>
+      <c r="G28" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="H28" s="18" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="46.15" x14ac:dyDescent="0.45">
+      <c r="A29" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="B29" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="C29" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="D29" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E29" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="F29" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="G29" s="18" t="s">
+        <v>136</v>
+      </c>
+      <c r="H29" s="18" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="46.15" x14ac:dyDescent="0.45">
+      <c r="A30" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="C30" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="D30" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E30" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="F30" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="G30" s="18" t="s">
+        <v>141</v>
+      </c>
+      <c r="H30" s="18" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
+      <c r="A31" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="B31" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="C31" s="18" t="s">
+        <v>144</v>
+      </c>
+      <c r="D31" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="E31" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="F31" s="18" t="s">
+        <v>145</v>
+      </c>
+      <c r="G31" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="H31" s="18" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="46.15" x14ac:dyDescent="0.45">
+      <c r="A32" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="B32" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="C32" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="D32" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="E32" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="F32" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="G32" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="H32" s="18" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="46.15" x14ac:dyDescent="0.45">
+      <c r="A33" s="18" t="s">
+        <v>153</v>
+      </c>
+      <c r="B33" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="C33" s="18" t="s">
+        <v>154</v>
+      </c>
+      <c r="D33" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="E33" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="F33" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="G33" s="18" t="s">
+        <v>155</v>
+      </c>
+      <c r="H33" s="18" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
+      <c r="A34" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="B34" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="C34" s="18" t="s">
+        <v>158</v>
+      </c>
+      <c r="D34" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E34" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="F34" s="18" t="s">
+        <v>197</v>
+      </c>
+      <c r="G34" s="18" t="s">
+        <v>159</v>
+      </c>
+      <c r="H34" s="18" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="46.15" x14ac:dyDescent="0.45">
+      <c r="A35" s="18" t="s">
+        <v>161</v>
+      </c>
+      <c r="B35" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="C35" s="18" t="s">
+        <v>162</v>
+      </c>
+      <c r="D35" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E35" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="F35" s="18" t="s">
+        <v>197</v>
+      </c>
+      <c r="G35" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="H35" s="18" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
+      <c r="A36" s="18" t="s">
+        <v>165</v>
+      </c>
+      <c r="B36" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="C36" s="18" t="s">
+        <v>166</v>
+      </c>
+      <c r="D36" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E36" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="F36" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="G36" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="H36" s="18" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="61.5" x14ac:dyDescent="0.45">
+      <c r="A37" s="18" t="s">
+        <v>169</v>
+      </c>
+      <c r="B37" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="C37" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="D37" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E37" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="F37" s="18" t="s">
+        <v>197</v>
+      </c>
+      <c r="G37" s="18" t="s">
+        <v>171</v>
+      </c>
+      <c r="H37" s="18" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A38" s="18" t="s">
+        <v>173</v>
+      </c>
+      <c r="B38" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="C38" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="D38" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E38" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="F38" s="18" t="s">
+        <v>198</v>
+      </c>
+      <c r="G38" s="18" t="s">
+        <v>175</v>
+      </c>
+      <c r="H38" s="18" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A39" s="18" t="s">
+        <v>177</v>
+      </c>
+      <c r="B39" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="C39" s="18" t="s">
+        <v>178</v>
+      </c>
+      <c r="D39" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E39" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="F39" s="18" t="s">
+        <v>197</v>
+      </c>
+      <c r="G39" s="18" t="s">
+        <v>180</v>
+      </c>
+      <c r="H39" s="18" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A40" s="18" t="s">
+        <v>182</v>
+      </c>
+      <c r="B40" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="C40" s="18" t="s">
+        <v>183</v>
+      </c>
+      <c r="D40" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E40" s="18" t="s">
+        <v>184</v>
+      </c>
+      <c r="F40" s="18" t="s">
+        <v>198</v>
+      </c>
+      <c r="G40" s="18" t="s">
+        <v>185</v>
+      </c>
+      <c r="H40" s="18" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="61.5" x14ac:dyDescent="0.45">
+      <c r="A41" s="18" t="s">
+        <v>187</v>
+      </c>
+      <c r="B41" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="C41" s="18" t="s">
+        <v>188</v>
+      </c>
+      <c r="D41" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="E41" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="F41" s="18" t="s">
+        <v>199</v>
+      </c>
+      <c r="G41" s="18" t="s">
+        <v>189</v>
+      </c>
+      <c r="H41" s="18" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="61.5" x14ac:dyDescent="0.45">
+      <c r="A42" s="18" t="s">
+        <v>191</v>
+      </c>
+      <c r="B42" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="C42" s="18" t="s">
+        <v>192</v>
+      </c>
+      <c r="D42" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="E42" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="F42" s="18" t="s">
+        <v>199</v>
+      </c>
+      <c r="G42" s="18" t="s">
+        <v>193</v>
+      </c>
+      <c r="H42" s="18" t="s">
+        <v>194</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B10:D10"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Product Details test case tab, cross-reference TC_PRODUCT_016 coverage
</commit_message>
<xml_diff>
--- a/test-cases/SauceDemo_TestCases.xlsx
+++ b/test-cases/SauceDemo_TestCases.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\saucedemo-playwright-pom\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88E1F1F0-E795-4C50-8453-7727C97E32E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A23C3D1-096A-43ED-9230-E0112DDC30A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
     <sheet name="Product Catalogue" sheetId="2" r:id="rId2"/>
+    <sheet name="Product Details" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="244">
   <si>
     <t>Field</t>
   </si>
@@ -772,6 +773,179 @@
   </si>
   <si>
     <t>Product: Backpack + Bike Light + Fleece Jacket (3 products)</t>
+  </si>
+  <si>
+    <t>Product Details</t>
+  </si>
+  <si>
+    <t>TS_PRODUCT_DETAILS_001</t>
+  </si>
+  <si>
+    <t>Verify product details displayed on the Product Details page</t>
+  </si>
+  <si>
+    <t>TS_PRODUCT_DETAILS_002</t>
+  </si>
+  <si>
+    <t>Verify navigation and cart functionality from the Product Details page</t>
+  </si>
+  <si>
+    <t>TS_PRODUCT_DETAILS_003</t>
+  </si>
+  <si>
+    <t>Verify product state is maintained when navigating between Product Details and other pages</t>
+  </si>
+  <si>
+    <t>Automated In</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_DETAILS_001</t>
+  </si>
+  <si>
+    <t>Verify product name is displayed on the Product Details page</t>
+  </si>
+  <si>
+    <t>Common Product Details Preconditions</t>
+  </si>
+  <si>
+    <t>1. Verify the product name.</t>
+  </si>
+  <si>
+    <t>The selected product name should be displayed correctly on the Product Details page.</t>
+  </si>
+  <si>
+    <t>Covered by TC_PRODUCT_016 (product.spec.js)</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_DETAILS_002</t>
+  </si>
+  <si>
+    <t>Verify product image, description, and price are displayed on the Product Details page</t>
+  </si>
+  <si>
+    <t>1. Verify the product image.
+2. Verify the product description.
+3. Verify the product price.</t>
+  </si>
+  <si>
+    <t>The selected product's image, description, and price should be displayed correctly.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_DETAILS_003</t>
+  </si>
+  <si>
+    <t>Verify product details match the selected product from the Product Listing page</t>
+  </si>
+  <si>
+    <t>1. Compare the displayed product details with
+the details captured from the Product Listing page.</t>
+  </si>
+  <si>
+    <t>Product name, description, and price on the Product Details page should match the selected product on the Product Listing page.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_DETAILS_004</t>
+  </si>
+  <si>
+    <t>Verify user can add a product to the cart from the Product Details page</t>
+  </si>
+  <si>
+    <t>1. Click Add to Cart.
+2. Verify the cart badge count.</t>
+  </si>
+  <si>
+    <t>The selected product should be added to the cart, and the cart badge should display 1.</t>
+  </si>
+  <si>
+    <t>product-details.spec.js</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_DETAILS_005</t>
+  </si>
+  <si>
+    <t>Verify user can remove a product from the cart from the Product Details page</t>
+  </si>
+  <si>
+    <t>Common Product Details Preconditions; 
+Selected product is already added to the cart</t>
+  </si>
+  <si>
+    <t>1. Click Remove.
+2. Verify the cart badge.</t>
+  </si>
+  <si>
+    <t>The selected product should be removed from the cart, and the cart badge should no longer display the product count.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_DETAILS_006</t>
+  </si>
+  <si>
+    <t>Verify Cart button navigates to the Cart page from the Product Details page</t>
+  </si>
+  <si>
+    <t>Common Product Details Preconditions; 
+Product is already added to the cart</t>
+  </si>
+  <si>
+    <t>1. Click the Cart icon.</t>
+  </si>
+  <si>
+    <t>User should be redirected successfully to the Cart page, and the added product should be displayed in the cart.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_DETAILS_007</t>
+  </si>
+  <si>
+    <t>Verify navigation back to Product Listing page from Product Details page</t>
+  </si>
+  <si>
+    <t>User is logged in and Product Details page is displayed</t>
+  </si>
+  <si>
+    <t>1. Navigate back to the Product Listing page.</t>
+  </si>
+  <si>
+    <t>User should be navigated successfully to the Product Listing page, and the product inventory should be displayed.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">Common Product Details Preconditions :
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>1. Sauce Demo application is accessible.
+2. User is logged in successfully.
+3. Product Listing page is displayed.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Common Test Steps:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>1. Select a product from the Product Listing page.
+2. Navigate to the Product Details page.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -932,7 +1106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -993,6 +1167,12 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2566,4 +2746,450 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{417D18E6-5B0B-4CD1-A071-EB56C7CA1658}">
+  <dimension ref="A1:I22"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="31.73046875" customWidth="1"/>
+    <col min="2" max="2" width="31.33203125" customWidth="1"/>
+    <col min="3" max="3" width="55.1328125" customWidth="1"/>
+    <col min="5" max="5" width="40.86328125" customWidth="1"/>
+    <col min="6" max="6" width="31.1328125" customWidth="1"/>
+    <col min="7" max="7" width="38.1328125" customWidth="1"/>
+    <col min="8" max="8" width="55.86328125" customWidth="1"/>
+    <col min="9" max="9" width="34" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="15" x14ac:dyDescent="0.4">
+      <c r="A1" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+    </row>
+    <row r="2" spans="1:9" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A2" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+    </row>
+    <row r="3" spans="1:9" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A3" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>200</v>
+      </c>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" s="20"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
+    </row>
+    <row r="5" spans="1:9" ht="15" x14ac:dyDescent="0.4">
+      <c r="A5" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="25"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20"/>
+      <c r="H5" s="20"/>
+      <c r="I5" s="20"/>
+    </row>
+    <row r="6" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A6" s="18" t="s">
+        <v>201</v>
+      </c>
+      <c r="B6" s="26" t="s">
+        <v>202</v>
+      </c>
+      <c r="C6" s="26"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="20"/>
+    </row>
+    <row r="7" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="B7" s="26" t="s">
+        <v>204</v>
+      </c>
+      <c r="C7" s="26"/>
+      <c r="D7" s="20"/>
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="20"/>
+      <c r="I7" s="20"/>
+    </row>
+    <row r="8" spans="1:9" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A8" s="18" t="s">
+        <v>205</v>
+      </c>
+      <c r="B8" s="26" t="s">
+        <v>206</v>
+      </c>
+      <c r="C8" s="26"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="20"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" s="20"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="20"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" s="20"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="20"/>
+      <c r="H10" s="20"/>
+      <c r="I10" s="20"/>
+    </row>
+    <row r="11" spans="1:9" ht="74.650000000000006" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A11" s="22" t="s">
+        <v>242</v>
+      </c>
+      <c r="B11" s="23"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="20"/>
+      <c r="F11" s="20"/>
+      <c r="G11" s="20"/>
+      <c r="H11" s="20"/>
+      <c r="I11" s="20"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A12" s="20"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="20"/>
+      <c r="H12" s="20"/>
+      <c r="I12" s="20"/>
+    </row>
+    <row r="13" spans="1:9" ht="70.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A13" s="22" t="s">
+        <v>243</v>
+      </c>
+      <c r="B13" s="23"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="20"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="20"/>
+      <c r="I13" s="20"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A14" s="20"/>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="20"/>
+      <c r="I14" s="20"/>
+    </row>
+    <row r="15" spans="1:9" ht="15" x14ac:dyDescent="0.4">
+      <c r="A15" s="24" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="E15" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="F15" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="G15" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="H15" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="I15" s="24" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="30.75" x14ac:dyDescent="0.45">
+      <c r="A16" s="18" t="s">
+        <v>208</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>201</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>209</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" s="18" t="s">
+        <v>210</v>
+      </c>
+      <c r="F16" s="18" t="s">
+        <v>197</v>
+      </c>
+      <c r="G16" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="H16" s="18" t="s">
+        <v>212</v>
+      </c>
+      <c r="I16" s="18" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="46.15" x14ac:dyDescent="0.45">
+      <c r="A17" s="18" t="s">
+        <v>214</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>201</v>
+      </c>
+      <c r="C17" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" s="18" t="s">
+        <v>210</v>
+      </c>
+      <c r="F17" s="18" t="s">
+        <v>197</v>
+      </c>
+      <c r="G17" s="18" t="s">
+        <v>216</v>
+      </c>
+      <c r="H17" s="18" t="s">
+        <v>217</v>
+      </c>
+      <c r="I17" s="18" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="61.5" x14ac:dyDescent="0.45">
+      <c r="A18" s="18" t="s">
+        <v>218</v>
+      </c>
+      <c r="B18" s="18" t="s">
+        <v>201</v>
+      </c>
+      <c r="C18" s="18" t="s">
+        <v>219</v>
+      </c>
+      <c r="D18" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E18" s="18" t="s">
+        <v>210</v>
+      </c>
+      <c r="F18" s="18" t="s">
+        <v>197</v>
+      </c>
+      <c r="G18" s="18" t="s">
+        <v>220</v>
+      </c>
+      <c r="H18" s="18" t="s">
+        <v>221</v>
+      </c>
+      <c r="I18" s="18" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="30.75" x14ac:dyDescent="0.45">
+      <c r="A19" s="18" t="s">
+        <v>222</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="C19" s="18" t="s">
+        <v>223</v>
+      </c>
+      <c r="D19" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E19" s="18" t="s">
+        <v>210</v>
+      </c>
+      <c r="F19" s="18" t="s">
+        <v>197</v>
+      </c>
+      <c r="G19" s="18" t="s">
+        <v>224</v>
+      </c>
+      <c r="H19" s="18" t="s">
+        <v>225</v>
+      </c>
+      <c r="I19" s="18" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="30.75" x14ac:dyDescent="0.45">
+      <c r="A20" s="18" t="s">
+        <v>227</v>
+      </c>
+      <c r="B20" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="C20" s="18" t="s">
+        <v>228</v>
+      </c>
+      <c r="D20" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E20" s="18" t="s">
+        <v>229</v>
+      </c>
+      <c r="F20" s="18" t="s">
+        <v>197</v>
+      </c>
+      <c r="G20" s="18" t="s">
+        <v>230</v>
+      </c>
+      <c r="H20" s="18" t="s">
+        <v>231</v>
+      </c>
+      <c r="I20" s="18" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="30.75" x14ac:dyDescent="0.45">
+      <c r="A21" s="18" t="s">
+        <v>232</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="C21" s="18" t="s">
+        <v>233</v>
+      </c>
+      <c r="D21" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E21" s="18" t="s">
+        <v>234</v>
+      </c>
+      <c r="F21" s="18" t="s">
+        <v>197</v>
+      </c>
+      <c r="G21" s="18" t="s">
+        <v>235</v>
+      </c>
+      <c r="H21" s="18" t="s">
+        <v>236</v>
+      </c>
+      <c r="I21" s="18" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="30.75" x14ac:dyDescent="0.45">
+      <c r="A22" s="18" t="s">
+        <v>237</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>205</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>238</v>
+      </c>
+      <c r="D22" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="E22" s="18" t="s">
+        <v>239</v>
+      </c>
+      <c r="F22" s="18" t="s">
+        <v>197</v>
+      </c>
+      <c r="G22" s="18" t="s">
+        <v>240</v>
+      </c>
+      <c r="H22" s="18" t="s">
+        <v>241</v>
+      </c>
+      <c r="I22" s="18" t="s">
+        <v>226</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A13:B13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: sync Cart module scenarios and test cases, consolidate scenario mapping
</commit_message>
<xml_diff>
--- a/test-cases/SauceDemo_TestCases.xlsx
+++ b/test-cases/SauceDemo_TestCases.xlsx
@@ -8,21 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\saucedemo-playwright-pom\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A23C3D1-096A-43ED-9230-E0112DDC30A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{126E94D9-3496-4CB3-9CC7-A40EAE3A31A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
     <sheet name="Product Catalogue" sheetId="2" r:id="rId2"/>
     <sheet name="Product Details" sheetId="3" r:id="rId3"/>
+    <sheet name="Cart" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="289">
   <si>
     <t>Field</t>
   </si>
@@ -947,12 +948,171 @@
 2. Navigate to the Product Details page.</t>
     </r>
   </si>
+  <si>
+    <t>Cart</t>
+  </si>
+  <si>
+    <t>TS_CART_001</t>
+  </si>
+  <si>
+    <t>Verify user can add a product to cart</t>
+  </si>
+  <si>
+    <t>TS_CART_002</t>
+  </si>
+  <si>
+    <t>Verify user can add multiple products to cart</t>
+  </si>
+  <si>
+    <t>TS_CART_003</t>
+  </si>
+  <si>
+    <t>Verify cart count updates after adding products</t>
+  </si>
+  <si>
+    <t>TS_CART_004</t>
+  </si>
+  <si>
+    <t>Verify selected products are displayed in cart</t>
+  </si>
+  <si>
+    <t>TS_CART_005</t>
+  </si>
+  <si>
+    <t>Verify product details in cart are correct</t>
+  </si>
+  <si>
+    <t>TS_CART_006</t>
+  </si>
+  <si>
+    <t>Verify user can remove products from cart</t>
+  </si>
+  <si>
+    <t>TS_CART_007</t>
+  </si>
+  <si>
+    <t>Verify cart count updates after removing products</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Common Cart Preconditions :
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>1. Sauce Demo application is accessible.
+2. User is logged in successfully.
+3. Product(s) are already added to the cart.
+4. User is on the Cart page.</t>
+    </r>
+  </si>
+  <si>
+    <t>TC_CART_001</t>
+  </si>
+  <si>
+    <t>Verify cart count is displayed correctly for added products</t>
+  </si>
+  <si>
+    <t>Common Cart Preconditions</t>
+  </si>
+  <si>
+    <t>Products: Sauce Labs Backpack, Sauce Labs Bike Light</t>
+  </si>
+  <si>
+    <t>1. Verify the cart badge count.</t>
+  </si>
+  <si>
+    <t>Cart badge should display the total number of products added to the cart.</t>
+  </si>
+  <si>
+    <t>TC_CART_002</t>
+  </si>
+  <si>
+    <t>Verify selected products are displayed in the cart</t>
+  </si>
+  <si>
+    <t>1. Verify each selected product is displayed in the cart.</t>
+  </si>
+  <si>
+    <t>All selected products should be displayed in the cart.</t>
+  </si>
+  <si>
+    <t>TC_CART_003</t>
+  </si>
+  <si>
+    <t>Verify product details displayed in the cart are correct</t>
+  </si>
+  <si>
+    <t>1. Verify the product name. 
+2. Verify the product description. 
+3. Verify the product price. 
+4. Verify the product quantity.</t>
+  </si>
+  <si>
+    <t>Product name, description, price, and quantity should be displayed correctly for the selected product.</t>
+  </si>
+  <si>
+    <t>TC_CART_004</t>
+  </si>
+  <si>
+    <t>Verify user can remove a product from the cart</t>
+  </si>
+  <si>
+    <t>1. Click Remove for the selected product. 
+2. Verify the product is no longer displayed in the cart.</t>
+  </si>
+  <si>
+    <t>The selected product should be removed successfully from the cart.</t>
+  </si>
+  <si>
+    <t>TC_CART_005</t>
+  </si>
+  <si>
+    <t>1. Click Remove for each selected product. 
+2. Verify the selected products are no longer displayed in the cart.</t>
+  </si>
+  <si>
+    <t>All selected products should be removed successfully from the cart.</t>
+  </si>
+  <si>
+    <t>TC_CART_006</t>
+  </si>
+  <si>
+    <t>Verify cart count is updated after removing a product</t>
+  </si>
+  <si>
+    <t>1. Note the current cart badge count. 
+2. Remove one product from the cart. 
+3. Verify the cart badge count.</t>
+  </si>
+  <si>
+    <t>Cart badge count should decrease by 1 after removing the product.</t>
+  </si>
+  <si>
+    <t>TC_CART_007</t>
+  </si>
+  <si>
+    <t>Verify cart count is updated after removing multiple products</t>
+  </si>
+  <si>
+    <t>1. Note the current cart badge count. 
+2. Remove the selected products. 
+3. Verify the cart badge count.</t>
+  </si>
+  <si>
+    <t>Cart badge count should decrease according to the number of products removed.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1012,6 +1172,12 @@
     </font>
     <font>
       <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
@@ -1106,7 +1272,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1124,25 +1290,11 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1156,12 +1308,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1173,6 +1319,35 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1447,7 +1622,7 @@
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -1461,10 +1636,10 @@
       <c r="A5" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="10"/>
+      <c r="C5" s="22"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
@@ -1475,10 +1650,10 @@
       <c r="A6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="10"/>
+      <c r="C6" s="22"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
@@ -1489,10 +1664,10 @@
       <c r="A7" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="10"/>
+      <c r="C7" s="22"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
@@ -1503,10 +1678,10 @@
       <c r="A8" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="10"/>
+      <c r="C8" s="22"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
@@ -1517,17 +1692,17 @@
       <c r="A9" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="10"/>
+      <c r="C9" s="22"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -1538,10 +1713,10 @@
       <c r="H10" s="2"/>
     </row>
     <row r="11" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="9" t="s">
+      <c r="A11" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="10"/>
+      <c r="B11" s="22"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
@@ -1549,7 +1724,7 @@
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -1560,10 +1735,10 @@
       <c r="H12" s="2"/>
     </row>
     <row r="13" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="9" t="s">
+      <c r="A13" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="10"/>
+      <c r="B13" s="22"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
@@ -1571,7 +1746,7 @@
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -1949,800 +2124,800 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15" x14ac:dyDescent="0.4">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="12" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="13" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" x14ac:dyDescent="0.35">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
     </row>
     <row r="6" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="25"/>
     </row>
     <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="B7" s="16" t="s">
+      <c r="B7" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="C7" s="16"/>
-      <c r="D7" s="16"/>
+      <c r="C7" s="25"/>
+      <c r="D7" s="25"/>
     </row>
     <row r="8" spans="1:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
+      <c r="C8" s="25"/>
+      <c r="D8" s="25"/>
     </row>
     <row r="9" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="B9" s="16" t="s">
+      <c r="B9" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
     </row>
     <row r="10" spans="1:8" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="25" t="s">
         <v>81</v>
       </c>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="25"/>
     </row>
     <row r="11" spans="1:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
+      <c r="C11" s="25"/>
+      <c r="D11" s="25"/>
     </row>
     <row r="12" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="B12" s="16" t="s">
+      <c r="B12" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="25"/>
     </row>
     <row r="13" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="B13" s="16" t="s">
+      <c r="B13" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
+      <c r="C13" s="25"/>
+      <c r="D13" s="25"/>
     </row>
     <row r="15" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="21" t="s">
+      <c r="A15" s="26" t="s">
         <v>195</v>
       </c>
-      <c r="B15" s="10"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="20"/>
+      <c r="B15" s="22"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="14"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A16" s="20"/>
-      <c r="B16" s="20"/>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="20"/>
+      <c r="A16" s="14"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="14"/>
+      <c r="H16" s="14"/>
     </row>
     <row r="17" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="19" t="s">
         <v>196</v>
       </c>
-      <c r="B17" s="23"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="20"/>
-      <c r="E17" s="20"/>
-      <c r="F17" s="20"/>
-      <c r="G17" s="20"/>
-      <c r="H17" s="20"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="14"/>
+      <c r="F17" s="14"/>
+      <c r="G17" s="14"/>
+      <c r="H17" s="14"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A18" s="20"/>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="20"/>
-      <c r="E18" s="20"/>
-      <c r="F18" s="20"/>
-      <c r="G18" s="20"/>
-      <c r="H18" s="20"/>
+      <c r="A18" s="14"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="14"/>
     </row>
     <row r="19" spans="1:8" ht="15" x14ac:dyDescent="0.4">
-      <c r="A19" s="24" t="s">
+      <c r="A19" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="24" t="s">
+      <c r="B19" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="24" t="s">
+      <c r="C19" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="D19" s="24" t="s">
+      <c r="D19" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="E19" s="24" t="s">
+      <c r="E19" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="F19" s="24" t="s">
+      <c r="F19" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="G19" s="24" t="s">
+      <c r="G19" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="H19" s="24" t="s">
+      <c r="H19" s="16" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
-      <c r="A20" s="18" t="s">
+    <row r="20" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A20" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="B20" s="18" t="s">
+      <c r="B20" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C20" s="18" t="s">
+      <c r="C20" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="D20" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E20" s="18" t="s">
+      <c r="E20" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="F20" s="18" t="s">
+      <c r="F20" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="G20" s="18" t="s">
+      <c r="G20" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="H20" s="18" t="s">
+      <c r="H20" s="12" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
-      <c r="A21" s="18" t="s">
+      <c r="A21" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="B21" s="18" t="s">
+      <c r="B21" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C21" s="18" t="s">
+      <c r="C21" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="D21" s="18" t="s">
+      <c r="D21" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E21" s="18" t="s">
+      <c r="E21" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="F21" s="18" t="s">
+      <c r="F21" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="G21" s="18" t="s">
+      <c r="G21" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="H21" s="18" t="s">
+      <c r="H21" s="12" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A22" s="18" t="s">
+      <c r="A22" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="B22" s="18" t="s">
+      <c r="B22" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C22" s="18" t="s">
+      <c r="C22" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="D22" s="18" t="s">
+      <c r="D22" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="E22" s="18" t="s">
+      <c r="E22" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="F22" s="18" t="s">
+      <c r="F22" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="G22" s="18" t="s">
+      <c r="G22" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="H22" s="18" t="s">
+      <c r="H22" s="12" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="76.900000000000006" x14ac:dyDescent="0.45">
-      <c r="A23" s="18" t="s">
+      <c r="A23" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="B23" s="18" t="s">
+      <c r="B23" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="C23" s="18" t="s">
+      <c r="C23" s="12" t="s">
         <v>103</v>
       </c>
-      <c r="D23" s="18" t="s">
+      <c r="D23" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E23" s="18" t="s">
+      <c r="E23" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="F23" s="18" t="s">
+      <c r="F23" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="G23" s="18" t="s">
+      <c r="G23" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="H23" s="18" t="s">
+      <c r="H23" s="12" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
-      <c r="A24" s="18" t="s">
+      <c r="A24" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="B24" s="18" t="s">
+      <c r="B24" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="C24" s="18" t="s">
+      <c r="C24" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="D24" s="18" t="s">
+      <c r="D24" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="E24" s="18" t="s">
+      <c r="E24" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="F24" s="18" t="s">
+      <c r="F24" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="G24" s="18" t="s">
+      <c r="G24" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="H24" s="18" t="s">
+      <c r="H24" s="12" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="46.15" x14ac:dyDescent="0.45">
-      <c r="A25" s="18" t="s">
+      <c r="A25" s="12" t="s">
         <v>113</v>
       </c>
-      <c r="B25" s="18" t="s">
+      <c r="B25" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="C25" s="18" t="s">
+      <c r="C25" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="D25" s="18" t="s">
+      <c r="D25" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="E25" s="18" t="s">
+      <c r="E25" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="F25" s="18" t="s">
+      <c r="F25" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="G25" s="18" t="s">
+      <c r="G25" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="H25" s="18" t="s">
+      <c r="H25" s="12" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
-      <c r="A26" s="18" t="s">
+      <c r="A26" s="12" t="s">
         <v>118</v>
       </c>
-      <c r="B26" s="18" t="s">
+      <c r="B26" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="C26" s="18" t="s">
+      <c r="C26" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="D26" s="18" t="s">
+      <c r="D26" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="E26" s="18" t="s">
+      <c r="E26" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="F26" s="18" t="s">
+      <c r="F26" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="G26" s="18" t="s">
+      <c r="G26" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="H26" s="18" t="s">
+      <c r="H26" s="12" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="46.15" x14ac:dyDescent="0.45">
-      <c r="A27" s="18" t="s">
+      <c r="A27" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="B27" s="18" t="s">
+      <c r="B27" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="C27" s="18" t="s">
+      <c r="C27" s="12" t="s">
         <v>124</v>
       </c>
-      <c r="D27" s="18" t="s">
+      <c r="D27" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E27" s="18" t="s">
+      <c r="E27" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="F27" s="18" t="s">
+      <c r="F27" s="12" t="s">
         <v>125</v>
       </c>
-      <c r="G27" s="18" t="s">
+      <c r="G27" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="H27" s="18" t="s">
+      <c r="H27" s="12" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="46.15" x14ac:dyDescent="0.45">
-      <c r="A28" s="18" t="s">
+      <c r="A28" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="B28" s="18" t="s">
+      <c r="B28" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="C28" s="18" t="s">
+      <c r="C28" s="12" t="s">
         <v>129</v>
       </c>
-      <c r="D28" s="18" t="s">
+      <c r="D28" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E28" s="18" t="s">
+      <c r="E28" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="F28" s="18" t="s">
+      <c r="F28" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="G28" s="18" t="s">
+      <c r="G28" s="12" t="s">
         <v>131</v>
       </c>
-      <c r="H28" s="18" t="s">
+      <c r="H28" s="12" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="46.15" x14ac:dyDescent="0.45">
-      <c r="A29" s="18" t="s">
+      <c r="A29" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="B29" s="18" t="s">
+      <c r="B29" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="C29" s="18" t="s">
+      <c r="C29" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="D29" s="18" t="s">
+      <c r="D29" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E29" s="18" t="s">
+      <c r="E29" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="F29" s="18" t="s">
+      <c r="F29" s="12" t="s">
         <v>135</v>
       </c>
-      <c r="G29" s="18" t="s">
+      <c r="G29" s="12" t="s">
         <v>136</v>
       </c>
-      <c r="H29" s="18" t="s">
+      <c r="H29" s="12" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="46.15" x14ac:dyDescent="0.45">
-      <c r="A30" s="18" t="s">
+      <c r="A30" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="B30" s="18" t="s">
+      <c r="B30" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="C30" s="18" t="s">
+      <c r="C30" s="12" t="s">
         <v>139</v>
       </c>
-      <c r="D30" s="18" t="s">
+      <c r="D30" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E30" s="18" t="s">
+      <c r="E30" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="F30" s="18" t="s">
+      <c r="F30" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="G30" s="18" t="s">
+      <c r="G30" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="H30" s="18" t="s">
+      <c r="H30" s="12" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
-      <c r="A31" s="18" t="s">
+      <c r="A31" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="B31" s="18" t="s">
+      <c r="B31" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="C31" s="18" t="s">
+      <c r="C31" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="D31" s="18" t="s">
+      <c r="D31" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="E31" s="18" t="s">
+      <c r="E31" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="F31" s="18" t="s">
+      <c r="F31" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="G31" s="18" t="s">
+      <c r="G31" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="H31" s="18" t="s">
+      <c r="H31" s="12" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="46.15" x14ac:dyDescent="0.45">
-      <c r="A32" s="18" t="s">
+      <c r="A32" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="B32" s="18" t="s">
+      <c r="B32" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="C32" s="18" t="s">
+      <c r="C32" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="D32" s="18" t="s">
+      <c r="D32" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="E32" s="18" t="s">
+      <c r="E32" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="F32" s="18" t="s">
+      <c r="F32" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="G32" s="18" t="s">
+      <c r="G32" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="H32" s="18" t="s">
+      <c r="H32" s="12" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="46.15" x14ac:dyDescent="0.45">
-      <c r="A33" s="18" t="s">
+      <c r="A33" s="12" t="s">
         <v>153</v>
       </c>
-      <c r="B33" s="18" t="s">
+      <c r="B33" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="C33" s="18" t="s">
+      <c r="C33" s="12" t="s">
         <v>154</v>
       </c>
-      <c r="D33" s="18" t="s">
+      <c r="D33" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="E33" s="18" t="s">
+      <c r="E33" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="F33" s="18" t="s">
+      <c r="F33" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="G33" s="18" t="s">
+      <c r="G33" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="H33" s="18" t="s">
+      <c r="H33" s="12" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
-      <c r="A34" s="18" t="s">
+      <c r="A34" s="12" t="s">
         <v>157</v>
       </c>
-      <c r="B34" s="18" t="s">
+      <c r="B34" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="C34" s="18" t="s">
+      <c r="C34" s="12" t="s">
         <v>158</v>
       </c>
-      <c r="D34" s="18" t="s">
+      <c r="D34" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E34" s="18" t="s">
+      <c r="E34" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="F34" s="18" t="s">
+      <c r="F34" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="G34" s="18" t="s">
+      <c r="G34" s="12" t="s">
         <v>159</v>
       </c>
-      <c r="H34" s="18" t="s">
+      <c r="H34" s="12" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="46.15" x14ac:dyDescent="0.45">
-      <c r="A35" s="18" t="s">
+      <c r="A35" s="12" t="s">
         <v>161</v>
       </c>
-      <c r="B35" s="18" t="s">
+      <c r="B35" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="C35" s="18" t="s">
+      <c r="C35" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="D35" s="18" t="s">
+      <c r="D35" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E35" s="18" t="s">
+      <c r="E35" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="F35" s="18" t="s">
+      <c r="F35" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="G35" s="18" t="s">
+      <c r="G35" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="H35" s="18" t="s">
+      <c r="H35" s="12" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
-      <c r="A36" s="18" t="s">
+      <c r="A36" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="B36" s="18" t="s">
+      <c r="B36" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="C36" s="18" t="s">
+      <c r="C36" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="D36" s="18" t="s">
+      <c r="D36" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E36" s="18" t="s">
+      <c r="E36" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="F36" s="18" t="s">
+      <c r="F36" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="G36" s="18" t="s">
+      <c r="G36" s="12" t="s">
         <v>167</v>
       </c>
-      <c r="H36" s="18" t="s">
+      <c r="H36" s="12" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="61.5" x14ac:dyDescent="0.45">
-      <c r="A37" s="18" t="s">
+      <c r="A37" s="12" t="s">
         <v>169</v>
       </c>
-      <c r="B37" s="18" t="s">
+      <c r="B37" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="C37" s="18" t="s">
+      <c r="C37" s="12" t="s">
         <v>170</v>
       </c>
-      <c r="D37" s="18" t="s">
+      <c r="D37" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E37" s="18" t="s">
+      <c r="E37" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="F37" s="18" t="s">
+      <c r="F37" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="G37" s="18" t="s">
+      <c r="G37" s="12" t="s">
         <v>171</v>
       </c>
-      <c r="H37" s="18" t="s">
+      <c r="H37" s="12" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="76.900000000000006" x14ac:dyDescent="0.45">
-      <c r="A38" s="18" t="s">
+      <c r="A38" s="12" t="s">
         <v>173</v>
       </c>
-      <c r="B38" s="18" t="s">
+      <c r="B38" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="C38" s="18" t="s">
+      <c r="C38" s="12" t="s">
         <v>174</v>
       </c>
-      <c r="D38" s="18" t="s">
+      <c r="D38" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E38" s="18" t="s">
+      <c r="E38" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="F38" s="18" t="s">
+      <c r="F38" s="12" t="s">
         <v>198</v>
       </c>
-      <c r="G38" s="18" t="s">
+      <c r="G38" s="12" t="s">
         <v>175</v>
       </c>
-      <c r="H38" s="18" t="s">
+      <c r="H38" s="12" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="76.900000000000006" x14ac:dyDescent="0.45">
-      <c r="A39" s="18" t="s">
+      <c r="A39" s="12" t="s">
         <v>177</v>
       </c>
-      <c r="B39" s="18" t="s">
+      <c r="B39" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="C39" s="18" t="s">
+      <c r="C39" s="12" t="s">
         <v>178</v>
       </c>
-      <c r="D39" s="18" t="s">
+      <c r="D39" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E39" s="18" t="s">
+      <c r="E39" s="12" t="s">
         <v>179</v>
       </c>
-      <c r="F39" s="18" t="s">
+      <c r="F39" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="G39" s="18" t="s">
+      <c r="G39" s="12" t="s">
         <v>180</v>
       </c>
-      <c r="H39" s="18" t="s">
+      <c r="H39" s="12" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="76.900000000000006" x14ac:dyDescent="0.45">
-      <c r="A40" s="18" t="s">
+      <c r="A40" s="12" t="s">
         <v>182</v>
       </c>
-      <c r="B40" s="18" t="s">
+      <c r="B40" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="C40" s="18" t="s">
+      <c r="C40" s="12" t="s">
         <v>183</v>
       </c>
-      <c r="D40" s="18" t="s">
+      <c r="D40" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E40" s="18" t="s">
+      <c r="E40" s="12" t="s">
         <v>184</v>
       </c>
-      <c r="F40" s="18" t="s">
+      <c r="F40" s="12" t="s">
         <v>198</v>
       </c>
-      <c r="G40" s="18" t="s">
+      <c r="G40" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="H40" s="18" t="s">
+      <c r="H40" s="12" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="61.5" x14ac:dyDescent="0.45">
-      <c r="A41" s="18" t="s">
+      <c r="A41" s="12" t="s">
         <v>187</v>
       </c>
-      <c r="B41" s="18" t="s">
+      <c r="B41" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="C41" s="18" t="s">
+      <c r="C41" s="12" t="s">
         <v>188</v>
       </c>
-      <c r="D41" s="18" t="s">
+      <c r="D41" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="E41" s="18" t="s">
+      <c r="E41" s="12" t="s">
         <v>179</v>
       </c>
-      <c r="F41" s="18" t="s">
+      <c r="F41" s="12" t="s">
         <v>199</v>
       </c>
-      <c r="G41" s="18" t="s">
+      <c r="G41" s="12" t="s">
         <v>189</v>
       </c>
-      <c r="H41" s="18" t="s">
+      <c r="H41" s="12" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="61.5" x14ac:dyDescent="0.45">
-      <c r="A42" s="18" t="s">
+      <c r="A42" s="12" t="s">
         <v>191</v>
       </c>
-      <c r="B42" s="18" t="s">
+      <c r="B42" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="C42" s="18" t="s">
+      <c r="C42" s="12" t="s">
         <v>192</v>
       </c>
-      <c r="D42" s="18" t="s">
+      <c r="D42" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="E42" s="18" t="s">
+      <c r="E42" s="12" t="s">
         <v>179</v>
       </c>
-      <c r="F42" s="18" t="s">
+      <c r="F42" s="12" t="s">
         <v>199</v>
       </c>
-      <c r="G42" s="18" t="s">
+      <c r="G42" s="12" t="s">
         <v>193</v>
       </c>
-      <c r="H42" s="18" t="s">
+      <c r="H42" s="12" t="s">
         <v>194</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B9:D9"/>
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="A15:B15"/>
     <mergeCell ref="A17:B17"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B10:D10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2764,431 +2939,865 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15" x14ac:dyDescent="0.4">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
     </row>
     <row r="2" spans="1:9" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
     </row>
     <row r="3" spans="1:9" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="13" t="s">
         <v>200</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
-      <c r="H3" s="20"/>
-      <c r="I3" s="20"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" s="20"/>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="20"/>
-      <c r="I4" s="20"/>
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="14"/>
     </row>
     <row r="5" spans="1:9" ht="15" x14ac:dyDescent="0.4">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="25" t="s">
+      <c r="B5" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="25"/>
-      <c r="D5" s="20"/>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20"/>
-      <c r="H5" s="20"/>
-      <c r="I5" s="20"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="14"/>
     </row>
     <row r="6" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="B6" s="26" t="s">
+      <c r="B6" s="18" t="s">
         <v>202</v>
       </c>
-      <c r="C6" s="26"/>
-      <c r="D6" s="20"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="20"/>
-      <c r="I6" s="20"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
     </row>
     <row r="7" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="12" t="s">
         <v>203</v>
       </c>
-      <c r="B7" s="26" t="s">
+      <c r="B7" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="C7" s="26"/>
-      <c r="D7" s="20"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="20"/>
-      <c r="H7" s="20"/>
-      <c r="I7" s="20"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="14"/>
     </row>
     <row r="8" spans="1:9" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="12" t="s">
         <v>205</v>
       </c>
-      <c r="B8" s="26" t="s">
+      <c r="B8" s="18" t="s">
         <v>206</v>
       </c>
-      <c r="C8" s="26"/>
-      <c r="D8" s="20"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="20"/>
-      <c r="H8" s="20"/>
-      <c r="I8" s="20"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+      <c r="I8" s="14"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A9" s="20"/>
-      <c r="B9" s="20"/>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="20"/>
-      <c r="I9" s="20"/>
+      <c r="A9" s="14"/>
+      <c r="B9" s="14"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="14"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A10" s="20"/>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="20"/>
-      <c r="H10" s="20"/>
-      <c r="I10" s="20"/>
+      <c r="A10" s="14"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
+      <c r="I10" s="14"/>
     </row>
     <row r="11" spans="1:9" ht="74.650000000000006" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="19" t="s">
         <v>242</v>
       </c>
-      <c r="B11" s="23"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20"/>
-      <c r="I11" s="20"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
+      <c r="H11" s="14"/>
+      <c r="I11" s="14"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A12" s="20"/>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="20"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="20"/>
-      <c r="H12" s="20"/>
-      <c r="I12" s="20"/>
+      <c r="A12" s="14"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="14"/>
+      <c r="G12" s="14"/>
+      <c r="H12" s="14"/>
+      <c r="I12" s="14"/>
     </row>
     <row r="13" spans="1:9" ht="70.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="22" t="s">
+      <c r="A13" s="19" t="s">
         <v>243</v>
       </c>
-      <c r="B13" s="23"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="20"/>
-      <c r="I13" s="20"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="14"/>
+      <c r="G13" s="14"/>
+      <c r="H13" s="14"/>
+      <c r="I13" s="14"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A14" s="20"/>
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="20"/>
-      <c r="I14" s="20"/>
+      <c r="A14" s="14"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="14"/>
+      <c r="H14" s="14"/>
+      <c r="I14" s="14"/>
     </row>
     <row r="15" spans="1:9" ht="15" x14ac:dyDescent="0.4">
-      <c r="A15" s="24" t="s">
+      <c r="A15" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="24" t="s">
+      <c r="B15" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="24" t="s">
+      <c r="C15" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="24" t="s">
+      <c r="D15" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="E15" s="24" t="s">
+      <c r="E15" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="F15" s="24" t="s">
+      <c r="F15" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="G15" s="24" t="s">
+      <c r="G15" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="H15" s="24" t="s">
+      <c r="H15" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="I15" s="24" t="s">
+      <c r="I15" s="16" t="s">
         <v>207</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="30.75" x14ac:dyDescent="0.45">
-      <c r="A16" s="18" t="s">
+      <c r="A16" s="12" t="s">
         <v>208</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="B16" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="C16" s="12" t="s">
         <v>209</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="D16" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E16" s="18" t="s">
+      <c r="E16" s="12" t="s">
         <v>210</v>
       </c>
-      <c r="F16" s="18" t="s">
+      <c r="F16" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="G16" s="18" t="s">
+      <c r="G16" s="12" t="s">
         <v>211</v>
       </c>
-      <c r="H16" s="18" t="s">
+      <c r="H16" s="12" t="s">
         <v>212</v>
       </c>
-      <c r="I16" s="18" t="s">
+      <c r="I16" s="12" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="46.15" x14ac:dyDescent="0.45">
-      <c r="A17" s="18" t="s">
+      <c r="A17" s="12" t="s">
         <v>214</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="B17" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="12" t="s">
         <v>215</v>
       </c>
-      <c r="D17" s="18" t="s">
+      <c r="D17" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E17" s="18" t="s">
+      <c r="E17" s="12" t="s">
         <v>210</v>
       </c>
-      <c r="F17" s="18" t="s">
+      <c r="F17" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="G17" s="18" t="s">
+      <c r="G17" s="12" t="s">
         <v>216</v>
       </c>
-      <c r="H17" s="18" t="s">
+      <c r="H17" s="12" t="s">
         <v>217</v>
       </c>
-      <c r="I17" s="18" t="s">
+      <c r="I17" s="12" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="61.5" x14ac:dyDescent="0.45">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="12" t="s">
         <v>218</v>
       </c>
-      <c r="B18" s="18" t="s">
+      <c r="B18" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="C18" s="18" t="s">
+      <c r="C18" s="12" t="s">
         <v>219</v>
       </c>
-      <c r="D18" s="18" t="s">
+      <c r="D18" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E18" s="18" t="s">
+      <c r="E18" s="12" t="s">
         <v>210</v>
       </c>
-      <c r="F18" s="18" t="s">
+      <c r="F18" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="G18" s="18" t="s">
+      <c r="G18" s="12" t="s">
         <v>220</v>
       </c>
-      <c r="H18" s="18" t="s">
+      <c r="H18" s="12" t="s">
         <v>221</v>
       </c>
-      <c r="I18" s="18" t="s">
+      <c r="I18" s="12" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="30.75" x14ac:dyDescent="0.45">
-      <c r="A19" s="18" t="s">
+      <c r="A19" s="12" t="s">
         <v>222</v>
       </c>
-      <c r="B19" s="18" t="s">
+      <c r="B19" s="12" t="s">
         <v>203</v>
       </c>
-      <c r="C19" s="18" t="s">
+      <c r="C19" s="12" t="s">
         <v>223</v>
       </c>
-      <c r="D19" s="18" t="s">
+      <c r="D19" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E19" s="18" t="s">
+      <c r="E19" s="12" t="s">
         <v>210</v>
       </c>
-      <c r="F19" s="18" t="s">
+      <c r="F19" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="G19" s="18" t="s">
+      <c r="G19" s="12" t="s">
         <v>224</v>
       </c>
-      <c r="H19" s="18" t="s">
+      <c r="H19" s="12" t="s">
         <v>225</v>
       </c>
-      <c r="I19" s="18" t="s">
+      <c r="I19" s="12" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="30.75" x14ac:dyDescent="0.45">
-      <c r="A20" s="18" t="s">
+      <c r="A20" s="12" t="s">
         <v>227</v>
       </c>
-      <c r="B20" s="18" t="s">
+      <c r="B20" s="12" t="s">
         <v>203</v>
       </c>
-      <c r="C20" s="18" t="s">
+      <c r="C20" s="12" t="s">
         <v>228</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="D20" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E20" s="18" t="s">
+      <c r="E20" s="12" t="s">
         <v>229</v>
       </c>
-      <c r="F20" s="18" t="s">
+      <c r="F20" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="G20" s="18" t="s">
+      <c r="G20" s="12" t="s">
         <v>230</v>
       </c>
-      <c r="H20" s="18" t="s">
+      <c r="H20" s="12" t="s">
         <v>231</v>
       </c>
-      <c r="I20" s="18" t="s">
+      <c r="I20" s="12" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="30.75" x14ac:dyDescent="0.45">
-      <c r="A21" s="18" t="s">
+      <c r="A21" s="12" t="s">
         <v>232</v>
       </c>
-      <c r="B21" s="18" t="s">
+      <c r="B21" s="12" t="s">
         <v>203</v>
       </c>
-      <c r="C21" s="18" t="s">
+      <c r="C21" s="12" t="s">
         <v>233</v>
       </c>
-      <c r="D21" s="18" t="s">
+      <c r="D21" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E21" s="18" t="s">
+      <c r="E21" s="12" t="s">
         <v>234</v>
       </c>
-      <c r="F21" s="18" t="s">
+      <c r="F21" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="G21" s="18" t="s">
+      <c r="G21" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="H21" s="18" t="s">
+      <c r="H21" s="12" t="s">
         <v>236</v>
       </c>
-      <c r="I21" s="18" t="s">
+      <c r="I21" s="12" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="30.75" x14ac:dyDescent="0.45">
-      <c r="A22" s="18" t="s">
+      <c r="A22" s="12" t="s">
         <v>237</v>
       </c>
-      <c r="B22" s="18" t="s">
+      <c r="B22" s="12" t="s">
         <v>205</v>
       </c>
-      <c r="C22" s="18" t="s">
+      <c r="C22" s="12" t="s">
         <v>238</v>
       </c>
-      <c r="D22" s="18" t="s">
+      <c r="D22" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="E22" s="18" t="s">
+      <c r="E22" s="12" t="s">
         <v>239</v>
       </c>
-      <c r="F22" s="18" t="s">
+      <c r="F22" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="G22" s="18" t="s">
+      <c r="G22" s="12" t="s">
         <v>240</v>
       </c>
-      <c r="H22" s="18" t="s">
+      <c r="H22" s="12" t="s">
         <v>241</v>
       </c>
-      <c r="I22" s="18" t="s">
+      <c r="I22" s="12" t="s">
         <v>226</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="A13:B13"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A13:B13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ADB7548-8D86-487D-9E9D-63B8B99D50DF}">
+  <dimension ref="A1:H23"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="14.73046875" customWidth="1"/>
+    <col min="2" max="2" width="14.9296875" customWidth="1"/>
+    <col min="3" max="3" width="51.59765625" customWidth="1"/>
+    <col min="4" max="4" width="7.9296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.33203125" customWidth="1"/>
+    <col min="6" max="6" width="35.1328125" customWidth="1"/>
+    <col min="7" max="7" width="35.9296875" customWidth="1"/>
+    <col min="8" max="8" width="75.73046875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="15" x14ac:dyDescent="0.4">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+    </row>
+    <row r="2" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A2" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+    </row>
+    <row r="3" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A3" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>244</v>
+      </c>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+    </row>
+    <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.4">
+      <c r="A5" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="17"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+    </row>
+    <row r="6" spans="1:8" ht="30.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A6" s="12" t="s">
+        <v>245</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>246</v>
+      </c>
+      <c r="C6" s="18"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+    </row>
+    <row r="7" spans="1:8" ht="46.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>248</v>
+      </c>
+      <c r="C7" s="18"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+    </row>
+    <row r="8" spans="1:8" ht="46.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A8" s="12" t="s">
+        <v>249</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>250</v>
+      </c>
+      <c r="C8" s="18"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+    </row>
+    <row r="9" spans="1:8" ht="46.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A9" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>252</v>
+      </c>
+      <c r="C9" s="18"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+    </row>
+    <row r="10" spans="1:8" ht="46.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A10" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>254</v>
+      </c>
+      <c r="C10" s="18"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
+    </row>
+    <row r="11" spans="1:8" ht="46.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A11" s="12" t="s">
+        <v>255</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>256</v>
+      </c>
+      <c r="C11" s="18"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
+      <c r="H11" s="14"/>
+    </row>
+    <row r="12" spans="1:8" ht="46.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A12" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>258</v>
+      </c>
+      <c r="C12" s="18"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="14"/>
+      <c r="G12" s="14"/>
+      <c r="H12" s="14"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" s="14"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="14"/>
+      <c r="G13" s="14"/>
+      <c r="H13" s="14"/>
+    </row>
+    <row r="14" spans="1:8" ht="195" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="15" t="s">
+        <v>259</v>
+      </c>
+      <c r="B14" s="15"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="14"/>
+      <c r="H14" s="14"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A15" s="14"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="14"/>
+    </row>
+    <row r="16" spans="1:8" ht="45" x14ac:dyDescent="0.4">
+      <c r="A16" s="29" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="29" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="29" t="s">
+        <v>21</v>
+      </c>
+      <c r="E16" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="F16" s="29" t="s">
+        <v>23</v>
+      </c>
+      <c r="G16" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="H16" s="29" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="153.75" x14ac:dyDescent="0.45">
+      <c r="A17" s="28" t="s">
+        <v>260</v>
+      </c>
+      <c r="B17" s="28" t="s">
+        <v>249</v>
+      </c>
+      <c r="C17" s="28" t="s">
+        <v>261</v>
+      </c>
+      <c r="D17" s="28" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" s="28" t="s">
+        <v>262</v>
+      </c>
+      <c r="F17" s="28" t="s">
+        <v>263</v>
+      </c>
+      <c r="G17" s="28" t="s">
+        <v>264</v>
+      </c>
+      <c r="H17" s="28" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="123" x14ac:dyDescent="0.45">
+      <c r="A18" s="28" t="s">
+        <v>266</v>
+      </c>
+      <c r="B18" s="28" t="s">
+        <v>251</v>
+      </c>
+      <c r="C18" s="28" t="s">
+        <v>267</v>
+      </c>
+      <c r="D18" s="28" t="s">
+        <v>28</v>
+      </c>
+      <c r="E18" s="28" t="s">
+        <v>262</v>
+      </c>
+      <c r="F18" s="28" t="s">
+        <v>263</v>
+      </c>
+      <c r="G18" s="28" t="s">
+        <v>268</v>
+      </c>
+      <c r="H18" s="28" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="261.39999999999998" x14ac:dyDescent="0.45">
+      <c r="A19" s="28" t="s">
+        <v>270</v>
+      </c>
+      <c r="B19" s="28" t="s">
+        <v>253</v>
+      </c>
+      <c r="C19" s="28" t="s">
+        <v>271</v>
+      </c>
+      <c r="D19" s="28" t="s">
+        <v>28</v>
+      </c>
+      <c r="E19" s="28" t="s">
+        <v>262</v>
+      </c>
+      <c r="F19" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="G19" s="28" t="s">
+        <v>272</v>
+      </c>
+      <c r="H19" s="28" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="184.5" x14ac:dyDescent="0.45">
+      <c r="A20" s="28" t="s">
+        <v>274</v>
+      </c>
+      <c r="B20" s="28" t="s">
+        <v>255</v>
+      </c>
+      <c r="C20" s="28" t="s">
+        <v>275</v>
+      </c>
+      <c r="D20" s="28" t="s">
+        <v>28</v>
+      </c>
+      <c r="E20" s="28" t="s">
+        <v>262</v>
+      </c>
+      <c r="F20" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="G20" s="28" t="s">
+        <v>276</v>
+      </c>
+      <c r="H20" s="28" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="215.25" x14ac:dyDescent="0.45">
+      <c r="A21" s="28" t="s">
+        <v>278</v>
+      </c>
+      <c r="B21" s="28" t="s">
+        <v>255</v>
+      </c>
+      <c r="C21" s="28" t="s">
+        <v>183</v>
+      </c>
+      <c r="D21" s="28" t="s">
+        <v>28</v>
+      </c>
+      <c r="E21" s="28" t="s">
+        <v>262</v>
+      </c>
+      <c r="F21" s="28" t="s">
+        <v>263</v>
+      </c>
+      <c r="G21" s="28" t="s">
+        <v>279</v>
+      </c>
+      <c r="H21" s="28" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="246" x14ac:dyDescent="0.45">
+      <c r="A22" s="28" t="s">
+        <v>281</v>
+      </c>
+      <c r="B22" s="28" t="s">
+        <v>257</v>
+      </c>
+      <c r="C22" s="28" t="s">
+        <v>282</v>
+      </c>
+      <c r="D22" s="28" t="s">
+        <v>28</v>
+      </c>
+      <c r="E22" s="28" t="s">
+        <v>262</v>
+      </c>
+      <c r="F22" s="28" t="s">
+        <v>263</v>
+      </c>
+      <c r="G22" s="28" t="s">
+        <v>283</v>
+      </c>
+      <c r="H22" s="28" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="230.65" x14ac:dyDescent="0.45">
+      <c r="A23" s="28" t="s">
+        <v>285</v>
+      </c>
+      <c r="B23" s="28" t="s">
+        <v>257</v>
+      </c>
+      <c r="C23" s="28" t="s">
+        <v>286</v>
+      </c>
+      <c r="D23" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="E23" s="28" t="s">
+        <v>262</v>
+      </c>
+      <c r="F23" s="28" t="s">
+        <v>263</v>
+      </c>
+      <c r="G23" s="28" t="s">
+        <v>287</v>
+      </c>
+      <c r="H23" s="28" t="s">
+        <v>288</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: add Checkout Info, Overview, and Complete test cases to Excel
</commit_message>
<xml_diff>
--- a/test-cases/SauceDemo_TestCases.xlsx
+++ b/test-cases/SauceDemo_TestCases.xlsx
@@ -8,22 +8,25 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\saucedemo-playwright-pom\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{126E94D9-3496-4CB3-9CC7-A40EAE3A31A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A25BC20-7664-4CE0-A0D1-CAF6A6DEF68B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
     <sheet name="Product Catalogue" sheetId="2" r:id="rId2"/>
     <sheet name="Product Details" sheetId="3" r:id="rId3"/>
     <sheet name="Cart" sheetId="4" r:id="rId4"/>
+    <sheet name="Checkout Info" sheetId="5" r:id="rId5"/>
+    <sheet name="Checkout Overview" sheetId="6" r:id="rId6"/>
+    <sheet name="Checkout Completion" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="714" uniqueCount="384">
   <si>
     <t>Field</t>
   </si>
@@ -955,46 +958,122 @@
     <t>TS_CART_001</t>
   </si>
   <si>
-    <t>Verify user can add a product to cart</t>
-  </si>
-  <si>
     <t>TS_CART_002</t>
   </si>
   <si>
-    <t>Verify user can add multiple products to cart</t>
-  </si>
-  <si>
     <t>TS_CART_003</t>
   </si>
   <si>
-    <t>Verify cart count updates after adding products</t>
-  </si>
-  <si>
     <t>TS_CART_004</t>
   </si>
   <si>
-    <t>Verify selected products are displayed in cart</t>
-  </si>
-  <si>
     <t>TS_CART_005</t>
   </si>
   <si>
-    <t>Verify product details in cart are correct</t>
-  </si>
-  <si>
-    <t>TS_CART_006</t>
-  </si>
-  <si>
-    <t>Verify user can remove products from cart</t>
-  </si>
-  <si>
-    <t>TS_CART_007</t>
-  </si>
-  <si>
-    <t>Verify cart count updates after removing products</t>
+    <t>TC_CART_001</t>
+  </si>
+  <si>
+    <t>Verify cart count is displayed correctly for added products</t>
+  </si>
+  <si>
+    <t>Common Cart Preconditions</t>
+  </si>
+  <si>
+    <t>Products: Sauce Labs Backpack, Sauce Labs Bike Light</t>
+  </si>
+  <si>
+    <t>1. Verify the cart badge count.</t>
+  </si>
+  <si>
+    <t>Cart badge should display the total number of products added to the cart.</t>
+  </si>
+  <si>
+    <t>TC_CART_002</t>
+  </si>
+  <si>
+    <t>Verify selected products are displayed in the cart</t>
+  </si>
+  <si>
+    <t>1. Verify each selected product is displayed in the cart.</t>
+  </si>
+  <si>
+    <t>All selected products should be displayed in the cart.</t>
+  </si>
+  <si>
+    <t>TC_CART_003</t>
+  </si>
+  <si>
+    <t>Verify product details displayed in the cart are correct</t>
+  </si>
+  <si>
+    <t>1. Verify the product name. 
+2. Verify the product description. 
+3. Verify the product price. 
+4. Verify the product quantity.</t>
+  </si>
+  <si>
+    <t>Product name, description, price, and quantity should be displayed correctly for the selected product.</t>
+  </si>
+  <si>
+    <t>TC_CART_004</t>
+  </si>
+  <si>
+    <t>Verify user can remove a product from the cart</t>
+  </si>
+  <si>
+    <t>1. Click Remove for the selected product. 
+2. Verify the product is no longer displayed in the cart.</t>
+  </si>
+  <si>
+    <t>The selected product should be removed successfully from the cart.</t>
+  </si>
+  <si>
+    <t>TC_CART_005</t>
+  </si>
+  <si>
+    <t>1. Click Remove for each selected product. 
+2. Verify the selected products are no longer displayed in the cart.</t>
+  </si>
+  <si>
+    <t>All selected products should be removed successfully from the cart.</t>
+  </si>
+  <si>
+    <t>TC_CART_006</t>
+  </si>
+  <si>
+    <t>Verify cart count is updated after removing a product</t>
+  </si>
+  <si>
+    <t>1. Note the current cart badge count. 
+2. Remove one product from the cart. 
+3. Verify the cart badge count.</t>
+  </si>
+  <si>
+    <t>Cart badge count should decrease by 1 after removing the product.</t>
+  </si>
+  <si>
+    <t>TC_CART_007</t>
+  </si>
+  <si>
+    <t>Verify cart count is updated after removing multiple products</t>
+  </si>
+  <si>
+    <t>1. Note the current cart badge count. 
+2. Remove the selected products. 
+3. Verify the cart badge count.</t>
+  </si>
+  <si>
+    <t>Cart badge count should decrease according to the number of products removed.</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
       <t xml:space="preserve">Common Cart Preconditions :
 </t>
     </r>
@@ -1002,8 +1081,8 @@
       <rPr>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
       </rPr>
       <t>1. Sauce Demo application is accessible.
 2. User is logged in successfully.
@@ -1012,107 +1091,409 @@
     </r>
   </si>
   <si>
-    <t>TC_CART_001</t>
-  </si>
-  <si>
-    <t>Verify cart count is displayed correctly for added products</t>
-  </si>
-  <si>
-    <t>Common Cart Preconditions</t>
-  </si>
-  <si>
-    <t>Products: Sauce Labs Backpack, Sauce Labs Bike Light</t>
-  </si>
-  <si>
-    <t>1. Verify the cart badge count.</t>
-  </si>
-  <si>
-    <t>Cart badge should display the total number of products added to the cart.</t>
-  </si>
-  <si>
-    <t>TC_CART_002</t>
-  </si>
-  <si>
-    <t>Verify selected products are displayed in the cart</t>
-  </si>
-  <si>
-    <t>1. Verify each selected product is displayed in the cart.</t>
-  </si>
-  <si>
-    <t>All selected products should be displayed in the cart.</t>
-  </si>
-  <si>
-    <t>TC_CART_003</t>
-  </si>
-  <si>
-    <t>Verify product details displayed in the cart are correct</t>
-  </si>
-  <si>
-    <t>1. Verify the product name. 
-2. Verify the product description. 
-3. Verify the product price. 
-4. Verify the product quantity.</t>
-  </si>
-  <si>
-    <t>Product name, description, price, and quantity should be displayed correctly for the selected product.</t>
-  </si>
-  <si>
-    <t>TC_CART_004</t>
-  </si>
-  <si>
-    <t>Verify user can remove a product from the cart</t>
-  </si>
-  <si>
-    <t>1. Click Remove for the selected product. 
-2. Verify the product is no longer displayed in the cart.</t>
-  </si>
-  <si>
-    <t>The selected product should be removed successfully from the cart.</t>
-  </si>
-  <si>
-    <t>TC_CART_005</t>
-  </si>
-  <si>
-    <t>1. Click Remove for each selected product. 
-2. Verify the selected products are no longer displayed in the cart.</t>
-  </si>
-  <si>
-    <t>All selected products should be removed successfully from the cart.</t>
-  </si>
-  <si>
-    <t>TC_CART_006</t>
-  </si>
-  <si>
-    <t>Verify cart count is updated after removing a product</t>
-  </si>
-  <si>
-    <t>1. Note the current cart badge count. 
-2. Remove one product from the cart. 
-3. Verify the cart badge count.</t>
-  </si>
-  <si>
-    <t>Cart badge count should decrease by 1 after removing the product.</t>
-  </si>
-  <si>
-    <t>TC_CART_007</t>
-  </si>
-  <si>
-    <t>Verify cart count is updated after removing multiple products</t>
-  </si>
-  <si>
-    <t>1. Note the current cart badge count. 
-2. Remove the selected products. 
-3. Verify the cart badge count.</t>
-  </si>
-  <si>
-    <t>Cart badge count should decrease according to the number of products removed.</t>
+    <t>Verify Continue Shopping button navigates back to inventory page</t>
+  </si>
+  <si>
+    <t>TC_CART_008</t>
+  </si>
+  <si>
+    <t>1. Click "Continue Shopping" button on the cart page.</t>
+  </si>
+  <si>
+    <t>User should be navigated back to the Products (inventory) page.</t>
+  </si>
+  <si>
+    <t>Verify Checkout button navigates to checkout information page</t>
+  </si>
+  <si>
+    <t>TC_CART_009</t>
+  </si>
+  <si>
+    <t>1. Click "Checkout" button on the cart page.</t>
+  </si>
+  <si>
+    <t>User should be navigated to the checkout step-one (information) page.</t>
+  </si>
+  <si>
+    <t>Verify products added to cart are reflected correctly (count and display)</t>
+  </si>
+  <si>
+    <t>Verify product details in cart are accurate</t>
+  </si>
+  <si>
+    <t>Verify products can be removed from cart</t>
+  </si>
+  <si>
+    <t>Verify cart badge count updates after removal</t>
+  </si>
+  <si>
+    <t>Verify cart page navigation actions</t>
+  </si>
+  <si>
+    <t>TS_CHECKOUT_COMPLETION_001</t>
+  </si>
+  <si>
+    <t>Verify order confirmation page and successful order completion message are displayed</t>
+  </si>
+  <si>
+    <t>TS_CHECKOUT_COMPLETION_002</t>
+  </si>
+  <si>
+    <t>Verify user can return to Products page after order completion</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_COMPLETION_001</t>
+  </si>
+  <si>
+    <t>1. Verify the Order Confirmation page. 
+2. Verify the confirmation message. 
+3. Verify the confirmation icon.</t>
+  </si>
+  <si>
+    <t>Order Confirmation page should be displayed with the appropriate
+successful order completion message and confirmation icon.</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_COMPLETION_002</t>
+  </si>
+  <si>
+    <t>1. Click Back Home. 
+2. Verify the Products page.</t>
+  </si>
+  <si>
+    <t>User should be navigated successfully to the Products page.</t>
+  </si>
+  <si>
+    <t>Checkout Overview</t>
+  </si>
+  <si>
+    <t>TS_CHECKOUT_OVERVIEW_001</t>
+  </si>
+  <si>
+    <t>Verify order summary details and price calculation</t>
+  </si>
+  <si>
+    <t>TS_CHECKOUT_OVERVIEW_002</t>
+  </si>
+  <si>
+    <t>Verify user can complete checkout successfully</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_OVERVIEW_001</t>
+  </si>
+  <si>
+    <t>Verify products and quantities are displayed correctly in the order summary</t>
+  </si>
+  <si>
+    <t>1. Enter valid customer information. 
+2. Click Continue. 
+3. Verify the selected product. 
+4. Verify the product quantity. 
+5. Verify the product price.</t>
+  </si>
+  <si>
+    <t>Order summary should display the correct product, quantity, and price.</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_OVERVIEW_002</t>
+  </si>
+  <si>
+    <t>Verify item total is calculated correctly</t>
+  </si>
+  <si>
+    <t>Product price and quantity</t>
+  </si>
+  <si>
+    <t>1. Note the product price and quantity. 
+2. Verify the Item Total.</t>
+  </si>
+  <si>
+    <t>Item Total should equal the sum of the prices of all products in the order.</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_OVERVIEW_003</t>
+  </si>
+  <si>
+    <t>Verify tax is calculated correctly</t>
+  </si>
+  <si>
+    <t>Product prices and displayed tax</t>
+  </si>
+  <si>
+    <t>1. Note the Item Total. 
+2. Note the displayed Tax. 
+3. Verify the tax amount.</t>
+  </si>
+  <si>
+    <t>Tax should be calculated correctly based on the applicable order amount.</t>
+  </si>
+  <si>
+    <t>Verify total amount is calculated correctly</t>
+  </si>
+  <si>
+    <t>Item Total and Tax</t>
+  </si>
+  <si>
+    <t>1. Note the Item Total. 
+2. Note the Tax. 
+3. Verify the Total.</t>
+  </si>
+  <si>
+    <t>Total should equal Item Total + Tax.</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_OVERVIEW_005</t>
+  </si>
+  <si>
+    <t>Valid customer information</t>
+  </si>
+  <si>
+    <t>1. Verify the order summary. 
+2. Click Finish. 
+3. Verify the order confirmation page.</t>
+  </si>
+  <si>
+    <t>Checkout Info</t>
+  </si>
+  <si>
+    <t>Verify user can navigate to and access the Checkout Information page</t>
+  </si>
+  <si>
+    <t>Verify customer information entry and mandatory field validation</t>
+  </si>
+  <si>
+    <t>Verify user can navigate back to Cart Page</t>
+  </si>
+  <si>
+    <t>Verify user can navigate to the Checkout Information page</t>
+  </si>
+  <si>
+    <t>1. Click Checkout.</t>
+  </si>
+  <si>
+    <t>User should be navigated successfully to the Checkout Information page.</t>
+  </si>
+  <si>
+    <t>Verify Checkout Information page displays required fields and controls</t>
+  </si>
+  <si>
+    <t>1. Verify First Name field. 
+2. Verify Last Name field. 
+3. Verify Postal Code field. 
+4. Verify Continue button. 
+5. Verify Cancel button.</t>
+  </si>
+  <si>
+    <t>Checkout Information page should display the required customer information fields and available action buttons.</t>
+  </si>
+  <si>
+    <t>Verify user can enter valid customer information</t>
+  </si>
+  <si>
+    <t>First Name: Harshitha 
+Last Name: Veeravalli
+Postal Code: 530001</t>
+  </si>
+  <si>
+    <t>1. Enter the first name.
+2. Enter the last name. 
+3. Enter the postal code.
+4. Click Continue Button</t>
+  </si>
+  <si>
+    <t>User should be able to enter valid customer information into the respective fields and re-direct to Checkout Overview Page</t>
+  </si>
+  <si>
+    <t>Verify validation when First Name is blank</t>
+  </si>
+  <si>
+    <t>First Name: -
+Last Name: Veeravalli
+Postal Code: 530001</t>
+  </si>
+  <si>
+    <t>1. Leave First Name blank. 
+2. Enter Last Name. 
+3. Enter Postal Code. 
+4. Click Continue Button.</t>
+  </si>
+  <si>
+    <t>Error message "Error: First Name is required" should be displayed and user should remain on the Checkout Information page.</t>
+  </si>
+  <si>
+    <t>Verify validation when Last Name is blank</t>
+  </si>
+  <si>
+    <t>First Name: Harshitha 
+Last Name: -
+Postal Code: 530001</t>
+  </si>
+  <si>
+    <t>1. Enter First Name. 
+2. Leave Last Name blank. 
+3. Enter Postal Code. 
+4. Click Continue Button.</t>
+  </si>
+  <si>
+    <t>Error message "Error: Last Name is required" should be displayed and user should remain on the Checkout Information page.</t>
+  </si>
+  <si>
+    <t>Verify validation when Postal Code is blank</t>
+  </si>
+  <si>
+    <t>First Name: Harshitha
+Last Name: Veeravalli
+Postal Code: -</t>
+  </si>
+  <si>
+    <t>1. Enter First Name. 
+2. Enter Last Name. 
+3. Leave Postal Code blank. 
+4. Click Continue Button.</t>
+  </si>
+  <si>
+    <t>Error message "Error: Postal Code is required" should be displayed and user should remain on the Checkout Information page.</t>
+  </si>
+  <si>
+    <t>Verify Cancel button returns user to the Cart page</t>
+  </si>
+  <si>
+    <t>User should be navigated successfully back to the Cart page.</t>
+  </si>
+  <si>
+    <t>1. Click Cancel Button.</t>
+  </si>
+  <si>
+    <t>User should be navigated to the Order Confirmation page.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Common Checkout Confirmation Preconditions :
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>1. Sauce Demo application is accessible.
+2. User is logged in successfully.
+3. Order has been completed successfully.
+4. Order Confirmation page is displayed.</t>
+    </r>
+  </si>
+  <si>
+    <t>Common Checkout Confirmation Preconditions</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Common Checkout Overview Preconditions :
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>1. Sauce Demo application is accessible.
+2. User is logged in successfully.
+3. Required product(s) are added to the cart.
+4. User is on the Cart page.</t>
+    </r>
+  </si>
+  <si>
+    <t>Common Checkout Overview Preconditions</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Common Checkout Info Preconditions :
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>1. Sauce Demo application is accessible.
+2. User is logged in successfully.
+3. Required product(s) are added to the cart.
+4. User is on the Cart page.</t>
+    </r>
+  </si>
+  <si>
+    <t>Common Checkout Info Preconditions</t>
+  </si>
+  <si>
+    <t>Common Checkout Info Preconditions
+Click Checkout Button</t>
+  </si>
+  <si>
+    <t>TS_CHECKOUT_INFO_001</t>
+  </si>
+  <si>
+    <t>TS_CHECKOUT_INFO_002</t>
+  </si>
+  <si>
+    <t>TS_CHECKOUT_INFO_003</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_INFO_002</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_INFO_003</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_INFO_004</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_INFO_005</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_INFO_006</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_INFO_007</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_INFO_001</t>
+  </si>
+  <si>
+    <t>Verify Cancel button returns user to the Product page</t>
+  </si>
+  <si>
+    <t>TS_CHECKOUT_OVERVIEW_003</t>
+  </si>
+  <si>
+    <t>Verify user can navigate back to Product Page</t>
+  </si>
+  <si>
+    <t>Common Checkout Overview Preconditions
+Click Cancel Button</t>
+  </si>
+  <si>
+    <t>User should be navigated successfully back to the Products page.</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_OVERVIEW_006</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_OVERVIEW_004</t>
+  </si>
+  <si>
+    <t>Checkout Completion</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1177,12 +1558,6 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1204,7 +1579,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -1268,6 +1643,32 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1308,22 +1709,19 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1337,17 +1735,20 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1636,10 +2037,10 @@
       <c r="A5" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="22"/>
+      <c r="C5" s="21"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
@@ -1650,10 +2051,10 @@
       <c r="A6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="22"/>
+      <c r="C6" s="21"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
@@ -1664,10 +2065,10 @@
       <c r="A7" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="22"/>
+      <c r="C7" s="21"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
@@ -1678,10 +2079,10 @@
       <c r="A8" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="B8" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="22"/>
+      <c r="C8" s="21"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
@@ -1692,10 +2093,10 @@
       <c r="A9" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="22"/>
+      <c r="C9" s="21"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
@@ -1713,10 +2114,10 @@
       <c r="H10" s="2"/>
     </row>
     <row r="11" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="21" t="s">
+      <c r="A11" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="22"/>
+      <c r="B11" s="21"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
@@ -1735,10 +2136,10 @@
       <c r="H12" s="2"/>
     </row>
     <row r="13" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="22"/>
+      <c r="B13" s="21"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
@@ -2151,97 +2552,97 @@
       <c r="A5" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
     </row>
     <row r="6" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B6" s="25" t="s">
+      <c r="B6" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="C6" s="25"/>
-      <c r="D6" s="25"/>
+      <c r="C6" s="24"/>
+      <c r="D6" s="24"/>
     </row>
     <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="C7" s="25"/>
-      <c r="D7" s="25"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="24"/>
     </row>
     <row r="8" spans="1:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="C8" s="25"/>
-      <c r="D8" s="25"/>
+      <c r="C8" s="24"/>
+      <c r="D8" s="24"/>
     </row>
     <row r="9" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="B9" s="25" t="s">
+      <c r="B9" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="C9" s="25"/>
-      <c r="D9" s="25"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
     </row>
     <row r="10" spans="1:8" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="B10" s="25" t="s">
+      <c r="B10" s="24" t="s">
         <v>81</v>
       </c>
-      <c r="C10" s="25"/>
-      <c r="D10" s="25"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
     </row>
     <row r="11" spans="1:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="B11" s="25" t="s">
+      <c r="B11" s="24" t="s">
         <v>83</v>
       </c>
-      <c r="C11" s="25"/>
-      <c r="D11" s="25"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="24"/>
     </row>
     <row r="12" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="B12" s="25" t="s">
+      <c r="B12" s="24" t="s">
         <v>85</v>
       </c>
-      <c r="C12" s="25"/>
-      <c r="D12" s="25"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="24"/>
     </row>
     <row r="13" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="B13" s="25" t="s">
+      <c r="B13" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="C13" s="25"/>
-      <c r="D13" s="25"/>
+      <c r="C13" s="24"/>
+      <c r="D13" s="24"/>
     </row>
     <row r="15" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="26" t="s">
         <v>195</v>
       </c>
-      <c r="B15" s="22"/>
+      <c r="B15" s="21"/>
       <c r="C15" s="14"/>
       <c r="D15" s="14"/>
       <c r="E15" s="14"/>
@@ -2260,10 +2661,10 @@
       <c r="H16" s="14"/>
     </row>
     <row r="17" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="19" t="s">
+      <c r="A17" s="27" t="s">
         <v>196</v>
       </c>
-      <c r="B17" s="20"/>
+      <c r="B17" s="28"/>
       <c r="C17" s="14"/>
       <c r="D17" s="14"/>
       <c r="E17" s="14"/>
@@ -2282,28 +2683,28 @@
       <c r="H18" s="14"/>
     </row>
     <row r="19" spans="1:8" ht="15" x14ac:dyDescent="0.4">
-      <c r="A19" s="16" t="s">
+      <c r="A19" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="16" t="s">
+      <c r="B19" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="16" t="s">
+      <c r="C19" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="D19" s="16" t="s">
+      <c r="D19" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="E19" s="16" t="s">
+      <c r="E19" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="F19" s="16" t="s">
+      <c r="F19" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="G19" s="16" t="s">
+      <c r="G19" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="H19" s="16" t="s">
+      <c r="H19" s="15" t="s">
         <v>25</v>
       </c>
     </row>
@@ -2907,17 +3308,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A17:B17"/>
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="B7:D7"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A17:B17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2998,10 +3399,10 @@
       <c r="A5" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="17"/>
+      <c r="C5" s="18"/>
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
       <c r="F5" s="14"/>
@@ -3013,10 +3414,10 @@
       <c r="A6" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="19" t="s">
         <v>202</v>
       </c>
-      <c r="C6" s="18"/>
+      <c r="C6" s="19"/>
       <c r="D6" s="14"/>
       <c r="E6" s="14"/>
       <c r="F6" s="14"/>
@@ -3028,10 +3429,10 @@
       <c r="A7" s="12" t="s">
         <v>203</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="19" t="s">
         <v>204</v>
       </c>
-      <c r="C7" s="18"/>
+      <c r="C7" s="19"/>
       <c r="D7" s="14"/>
       <c r="E7" s="14"/>
       <c r="F7" s="14"/>
@@ -3043,10 +3444,10 @@
       <c r="A8" s="12" t="s">
         <v>205</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="19" t="s">
         <v>206</v>
       </c>
-      <c r="C8" s="18"/>
+      <c r="C8" s="19"/>
       <c r="D8" s="14"/>
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
@@ -3077,10 +3478,10 @@
       <c r="I10" s="14"/>
     </row>
     <row r="11" spans="1:9" ht="74.650000000000006" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="27" t="s">
         <v>242</v>
       </c>
-      <c r="B11" s="20"/>
+      <c r="B11" s="28"/>
       <c r="C11" s="14"/>
       <c r="D11" s="14"/>
       <c r="E11" s="14"/>
@@ -3101,10 +3502,10 @@
       <c r="I12" s="14"/>
     </row>
     <row r="13" spans="1:9" ht="70.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="27" t="s">
         <v>243</v>
       </c>
-      <c r="B13" s="20"/>
+      <c r="B13" s="28"/>
       <c r="C13" s="14"/>
       <c r="D13" s="14"/>
       <c r="E13" s="14"/>
@@ -3125,31 +3526,31 @@
       <c r="I14" s="14"/>
     </row>
     <row r="15" spans="1:9" ht="15" x14ac:dyDescent="0.4">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="16" t="s">
+      <c r="B15" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="C15" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="16" t="s">
+      <c r="D15" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="E15" s="16" t="s">
+      <c r="E15" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="F15" s="16" t="s">
+      <c r="F15" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="G15" s="16" t="s">
+      <c r="G15" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="H15" s="16" t="s">
+      <c r="H15" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="I15" s="16" t="s">
+      <c r="I15" s="15" t="s">
         <v>207</v>
       </c>
     </row>
@@ -3375,12 +3776,12 @@
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.73046875" customWidth="1"/>
-    <col min="2" max="2" width="14.9296875" customWidth="1"/>
-    <col min="3" max="3" width="51.59765625" customWidth="1"/>
+    <col min="2" max="2" width="31.73046875" customWidth="1"/>
+    <col min="3" max="3" width="59.46484375" customWidth="1"/>
     <col min="4" max="4" width="7.9296875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="33.33203125" customWidth="1"/>
     <col min="6" max="6" width="35.1328125" customWidth="1"/>
-    <col min="7" max="7" width="35.9296875" customWidth="1"/>
+    <col min="7" max="7" width="50.33203125" customWidth="1"/>
     <col min="8" max="8" width="75.73046875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3436,112 +3837,106 @@
       <c r="G4" s="14"/>
       <c r="H4" s="14"/>
     </row>
-    <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:8" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="17"/>
+      <c r="C5" s="18"/>
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
       <c r="F5" s="14"/>
       <c r="G5" s="14"/>
       <c r="H5" s="14"/>
     </row>
-    <row r="6" spans="1:8" ht="30.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="12" t="s">
         <v>245</v>
       </c>
-      <c r="B6" s="18" t="s">
-        <v>246</v>
-      </c>
-      <c r="C6" s="18"/>
+      <c r="B6" s="19" t="s">
+        <v>288</v>
+      </c>
+      <c r="C6" s="19"/>
       <c r="D6" s="14"/>
       <c r="E6" s="14"/>
       <c r="F6" s="14"/>
       <c r="G6" s="14"/>
       <c r="H6" s="14"/>
     </row>
-    <row r="7" spans="1:8" ht="46.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:8" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="B7" s="18" t="s">
-        <v>248</v>
-      </c>
-      <c r="C7" s="18"/>
+        <v>246</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>289</v>
+      </c>
+      <c r="C7" s="19"/>
       <c r="D7" s="14"/>
       <c r="E7" s="14"/>
       <c r="F7" s="14"/>
       <c r="G7" s="14"/>
       <c r="H7" s="14"/>
     </row>
-    <row r="8" spans="1:8" ht="46.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:8" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="12" t="s">
-        <v>249</v>
-      </c>
-      <c r="B8" s="18" t="s">
-        <v>250</v>
-      </c>
-      <c r="C8" s="18"/>
+        <v>247</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>290</v>
+      </c>
+      <c r="C8" s="19"/>
       <c r="D8" s="14"/>
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
       <c r="G8" s="14"/>
       <c r="H8" s="14"/>
     </row>
-    <row r="9" spans="1:8" ht="46.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="12" t="s">
-        <v>251</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>252</v>
-      </c>
-      <c r="C9" s="18"/>
+        <v>248</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>291</v>
+      </c>
+      <c r="C9" s="19"/>
       <c r="D9" s="14"/>
       <c r="E9" s="14"/>
       <c r="F9" s="14"/>
       <c r="G9" s="14"/>
       <c r="H9" s="14"/>
     </row>
-    <row r="10" spans="1:8" ht="46.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:8" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="12" t="s">
-        <v>253</v>
-      </c>
-      <c r="B10" s="18" t="s">
-        <v>254</v>
-      </c>
-      <c r="C10" s="18"/>
+        <v>249</v>
+      </c>
+      <c r="B10" s="19" t="s">
+        <v>292</v>
+      </c>
+      <c r="C10" s="19"/>
       <c r="D10" s="14"/>
       <c r="E10" s="14"/>
       <c r="F10" s="14"/>
       <c r="G10" s="14"/>
       <c r="H10" s="14"/>
     </row>
-    <row r="11" spans="1:8" ht="46.15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="12" t="s">
-        <v>255</v>
-      </c>
-      <c r="B11" s="18" t="s">
-        <v>256</v>
-      </c>
-      <c r="C11" s="18"/>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" s="14"/>
+      <c r="B11" s="14"/>
+      <c r="C11" s="14"/>
       <c r="D11" s="14"/>
       <c r="E11" s="14"/>
       <c r="F11" s="14"/>
       <c r="G11" s="14"/>
       <c r="H11" s="14"/>
     </row>
-    <row r="12" spans="1:8" ht="46.15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="12" t="s">
-        <v>257</v>
-      </c>
-      <c r="B12" s="18" t="s">
-        <v>258</v>
-      </c>
-      <c r="C12" s="18"/>
+    <row r="12" spans="1:8" ht="97.9" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A12" s="16" t="s">
+        <v>279</v>
+      </c>
+      <c r="B12" s="17"/>
+      <c r="C12" s="14"/>
       <c r="D12" s="14"/>
       <c r="E12" s="14"/>
       <c r="F12" s="14"/>
@@ -3558,240 +3953,269 @@
       <c r="G13" s="14"/>
       <c r="H13" s="14"/>
     </row>
-    <row r="14" spans="1:8" ht="195" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:8" ht="15" x14ac:dyDescent="0.4">
       <c r="A14" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E14" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="F14" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="G14" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="H14" s="15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
+      <c r="A15" s="12" t="s">
+        <v>250</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>245</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>252</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="G15" s="12" t="s">
+        <v>254</v>
+      </c>
+      <c r="H15" s="12" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
+      <c r="A16" s="12" t="s">
+        <v>256</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>245</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>252</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="G16" s="12" t="s">
+        <v>258</v>
+      </c>
+      <c r="H16" s="12" t="s">
         <v>259</v>
       </c>
-      <c r="B14" s="15"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A15" s="14"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
-    </row>
-    <row r="16" spans="1:8" ht="45" x14ac:dyDescent="0.4">
-      <c r="A16" s="29" t="s">
-        <v>18</v>
-      </c>
-      <c r="B16" s="29" t="s">
-        <v>6</v>
-      </c>
-      <c r="C16" s="29" t="s">
-        <v>20</v>
-      </c>
-      <c r="D16" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="E16" s="29" t="s">
-        <v>22</v>
-      </c>
-      <c r="F16" s="29" t="s">
-        <v>23</v>
-      </c>
-      <c r="G16" s="29" t="s">
-        <v>24</v>
-      </c>
-      <c r="H16" s="29" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="153.75" x14ac:dyDescent="0.45">
-      <c r="A17" s="28" t="s">
+    </row>
+    <row r="17" spans="1:8" ht="61.5" x14ac:dyDescent="0.45">
+      <c r="A17" s="12" t="s">
         <v>260</v>
       </c>
-      <c r="B17" s="28" t="s">
+      <c r="B17" s="12" t="s">
+        <v>246</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>261</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>252</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="G17" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="H17" s="12" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
+      <c r="A18" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>252</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="G18" s="12" t="s">
+        <v>266</v>
+      </c>
+      <c r="H18" s="12" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="46.15" x14ac:dyDescent="0.45">
+      <c r="A19" s="12" t="s">
+        <v>268</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>252</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="G19" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="H19" s="12" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="46.15" x14ac:dyDescent="0.45">
+      <c r="A20" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>272</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>252</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="G20" s="12" t="s">
+        <v>273</v>
+      </c>
+      <c r="H20" s="12" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="46.15" x14ac:dyDescent="0.45">
+      <c r="A21" s="12" t="s">
+        <v>275</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>276</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E21" s="12" t="s">
+        <v>252</v>
+      </c>
+      <c r="F21" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="G21" s="12" t="s">
+        <v>277</v>
+      </c>
+      <c r="H21" s="12" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A22" s="12" t="s">
+        <v>281</v>
+      </c>
+      <c r="B22" s="12" t="s">
         <v>249</v>
       </c>
-      <c r="C17" s="28" t="s">
-        <v>261</v>
-      </c>
-      <c r="D17" s="28" t="s">
+      <c r="C22" s="12" t="s">
+        <v>280</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>252</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="G22" s="12" t="s">
+        <v>282</v>
+      </c>
+      <c r="H22" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A23" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>249</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>284</v>
+      </c>
+      <c r="D23" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E17" s="28" t="s">
-        <v>262</v>
-      </c>
-      <c r="F17" s="28" t="s">
-        <v>263</v>
-      </c>
-      <c r="G17" s="28" t="s">
-        <v>264</v>
-      </c>
-      <c r="H17" s="28" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="123" x14ac:dyDescent="0.45">
-      <c r="A18" s="28" t="s">
-        <v>266</v>
-      </c>
-      <c r="B18" s="28" t="s">
-        <v>251</v>
-      </c>
-      <c r="C18" s="28" t="s">
-        <v>267</v>
-      </c>
-      <c r="D18" s="28" t="s">
-        <v>28</v>
-      </c>
-      <c r="E18" s="28" t="s">
-        <v>262</v>
-      </c>
-      <c r="F18" s="28" t="s">
-        <v>263</v>
-      </c>
-      <c r="G18" s="28" t="s">
-        <v>268</v>
-      </c>
-      <c r="H18" s="28" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="261.39999999999998" x14ac:dyDescent="0.45">
-      <c r="A19" s="28" t="s">
-        <v>270</v>
-      </c>
-      <c r="B19" s="28" t="s">
-        <v>253</v>
-      </c>
-      <c r="C19" s="28" t="s">
-        <v>271</v>
-      </c>
-      <c r="D19" s="28" t="s">
-        <v>28</v>
-      </c>
-      <c r="E19" s="28" t="s">
-        <v>262</v>
-      </c>
-      <c r="F19" s="28" t="s">
+      <c r="E23" s="12" t="s">
+        <v>252</v>
+      </c>
+      <c r="F23" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="G19" s="28" t="s">
-        <v>272</v>
-      </c>
-      <c r="H19" s="28" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="184.5" x14ac:dyDescent="0.45">
-      <c r="A20" s="28" t="s">
-        <v>274</v>
-      </c>
-      <c r="B20" s="28" t="s">
-        <v>255</v>
-      </c>
-      <c r="C20" s="28" t="s">
-        <v>275</v>
-      </c>
-      <c r="D20" s="28" t="s">
-        <v>28</v>
-      </c>
-      <c r="E20" s="28" t="s">
-        <v>262</v>
-      </c>
-      <c r="F20" s="28" t="s">
-        <v>150</v>
-      </c>
-      <c r="G20" s="28" t="s">
-        <v>276</v>
-      </c>
-      <c r="H20" s="28" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="215.25" x14ac:dyDescent="0.45">
-      <c r="A21" s="28" t="s">
-        <v>278</v>
-      </c>
-      <c r="B21" s="28" t="s">
-        <v>255</v>
-      </c>
-      <c r="C21" s="28" t="s">
-        <v>183</v>
-      </c>
-      <c r="D21" s="28" t="s">
-        <v>28</v>
-      </c>
-      <c r="E21" s="28" t="s">
-        <v>262</v>
-      </c>
-      <c r="F21" s="28" t="s">
-        <v>263</v>
-      </c>
-      <c r="G21" s="28" t="s">
-        <v>279</v>
-      </c>
-      <c r="H21" s="28" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="246" x14ac:dyDescent="0.45">
-      <c r="A22" s="28" t="s">
-        <v>281</v>
-      </c>
-      <c r="B22" s="28" t="s">
-        <v>257</v>
-      </c>
-      <c r="C22" s="28" t="s">
-        <v>282</v>
-      </c>
-      <c r="D22" s="28" t="s">
-        <v>28</v>
-      </c>
-      <c r="E22" s="28" t="s">
-        <v>262</v>
-      </c>
-      <c r="F22" s="28" t="s">
-        <v>263</v>
-      </c>
-      <c r="G22" s="28" t="s">
-        <v>283</v>
-      </c>
-      <c r="H22" s="28" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="230.65" x14ac:dyDescent="0.45">
-      <c r="A23" s="28" t="s">
-        <v>285</v>
-      </c>
-      <c r="B23" s="28" t="s">
-        <v>257</v>
-      </c>
-      <c r="C23" s="28" t="s">
+      <c r="G23" s="12" t="s">
         <v>286</v>
       </c>
-      <c r="D23" s="28" t="s">
-        <v>35</v>
-      </c>
-      <c r="E23" s="28" t="s">
-        <v>262</v>
-      </c>
-      <c r="F23" s="28" t="s">
-        <v>263</v>
-      </c>
-      <c r="G23" s="28" t="s">
+      <c r="H23" s="12" t="s">
         <v>287</v>
       </c>
-      <c r="H23" s="28" t="s">
-        <v>288</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
+  <mergeCells count="7">
+    <mergeCell ref="A12:B12"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B7:C7"/>
@@ -3801,4 +4225,959 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50180D44-7ECF-4A12-997E-231837275F7B}">
+  <dimension ref="A1:H19"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="29.6640625" customWidth="1"/>
+    <col min="2" max="2" width="27.6640625" customWidth="1"/>
+    <col min="3" max="3" width="54.265625" customWidth="1"/>
+    <col min="5" max="5" width="41.796875" customWidth="1"/>
+    <col min="6" max="6" width="21.86328125" customWidth="1"/>
+    <col min="7" max="7" width="40.86328125" customWidth="1"/>
+    <col min="8" max="8" width="68" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="15" x14ac:dyDescent="0.4">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+    </row>
+    <row r="2" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A2" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+    </row>
+    <row r="3" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A3" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>329</v>
+      </c>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+    </row>
+    <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="18"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+    </row>
+    <row r="6" spans="1:8" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A6" s="12" t="s">
+        <v>366</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>330</v>
+      </c>
+      <c r="C6" s="19"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+    </row>
+    <row r="7" spans="1:8" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="12" t="s">
+        <v>367</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>331</v>
+      </c>
+      <c r="C7" s="19"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+    </row>
+    <row r="8" spans="1:8" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A8" s="12" t="s">
+        <v>368</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>332</v>
+      </c>
+      <c r="C8" s="19"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+    </row>
+    <row r="9" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="14"/>
+      <c r="B9" s="14"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+    </row>
+    <row r="10" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A10" s="27" t="s">
+        <v>363</v>
+      </c>
+      <c r="B10" s="28"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" s="14"/>
+      <c r="B11" s="14"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
+      <c r="H11" s="14"/>
+    </row>
+    <row r="12" spans="1:8" ht="15" x14ac:dyDescent="0.4">
+      <c r="A12" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="G12" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="H12" s="15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A13" s="12" t="s">
+        <v>375</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>366</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>364</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="G13" s="12" t="s">
+        <v>334</v>
+      </c>
+      <c r="H13" s="12" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A14" s="12" t="s">
+        <v>369</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>366</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>336</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>365</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="G14" s="12" t="s">
+        <v>337</v>
+      </c>
+      <c r="H14" s="12" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="61.5" x14ac:dyDescent="0.45">
+      <c r="A15" s="12" t="s">
+        <v>370</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>367</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>339</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>365</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>340</v>
+      </c>
+      <c r="G15" s="12" t="s">
+        <v>341</v>
+      </c>
+      <c r="H15" s="12" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="61.5" x14ac:dyDescent="0.45">
+      <c r="A16" s="12" t="s">
+        <v>371</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>367</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>343</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>365</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>344</v>
+      </c>
+      <c r="G16" s="12" t="s">
+        <v>345</v>
+      </c>
+      <c r="H16" s="12" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="61.5" x14ac:dyDescent="0.45">
+      <c r="A17" s="12" t="s">
+        <v>372</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>367</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>347</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>365</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>348</v>
+      </c>
+      <c r="G17" s="12" t="s">
+        <v>349</v>
+      </c>
+      <c r="H17" s="12" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="61.5" x14ac:dyDescent="0.45">
+      <c r="A18" s="12" t="s">
+        <v>373</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>367</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>365</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>352</v>
+      </c>
+      <c r="G18" s="12" t="s">
+        <v>353</v>
+      </c>
+      <c r="H18" s="12" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
+      <c r="A19" s="12" t="s">
+        <v>374</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>368</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>355</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>365</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="G19" s="12" t="s">
+        <v>357</v>
+      </c>
+      <c r="H19" s="12" t="s">
+        <v>356</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="A10:B10"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78B373D9-AB81-4185-A302-5F5807E08B32}">
+  <dimension ref="A1:H20"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="34.19921875" customWidth="1"/>
+    <col min="2" max="2" width="34.1328125" customWidth="1"/>
+    <col min="3" max="3" width="50.6640625" customWidth="1"/>
+    <col min="5" max="5" width="43.796875" customWidth="1"/>
+    <col min="6" max="6" width="20.46484375" customWidth="1"/>
+    <col min="7" max="7" width="36.9296875" customWidth="1"/>
+    <col min="8" max="8" width="54.3984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="15" x14ac:dyDescent="0.4">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+    </row>
+    <row r="2" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A2" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+    </row>
+    <row r="3" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A3" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>303</v>
+      </c>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+    </row>
+    <row r="5" spans="1:8" ht="15" x14ac:dyDescent="0.4">
+      <c r="A5" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="18"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+    </row>
+    <row r="6" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A6" s="12" t="s">
+        <v>304</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>305</v>
+      </c>
+      <c r="C6" s="19"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+    </row>
+    <row r="7" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A7" s="12" t="s">
+        <v>306</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>307</v>
+      </c>
+      <c r="C7" s="19"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+    </row>
+    <row r="8" spans="1:8" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A8" s="12" t="s">
+        <v>377</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>378</v>
+      </c>
+      <c r="C8" s="19"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" s="14"/>
+      <c r="B9" s="14"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+    </row>
+    <row r="10" spans="1:8" ht="96.4" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A10" s="27" t="s">
+        <v>361</v>
+      </c>
+      <c r="B10" s="28"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" s="14"/>
+      <c r="B11" s="14"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
+      <c r="H11" s="14"/>
+    </row>
+    <row r="12" spans="1:8" ht="15" x14ac:dyDescent="0.4">
+      <c r="A12" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="G12" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="H12" s="15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A13" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>304</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>309</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>362</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="G13" s="12" t="s">
+        <v>310</v>
+      </c>
+      <c r="H13" s="12" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
+      <c r="A14" s="12" t="s">
+        <v>312</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>304</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>313</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>362</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>314</v>
+      </c>
+      <c r="G14" s="12" t="s">
+        <v>315</v>
+      </c>
+      <c r="H14" s="12" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="46.15" x14ac:dyDescent="0.45">
+      <c r="A15" s="12" t="s">
+        <v>317</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>304</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>318</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>362</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>319</v>
+      </c>
+      <c r="G15" s="12" t="s">
+        <v>320</v>
+      </c>
+      <c r="H15" s="12" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="46.15" x14ac:dyDescent="0.45">
+      <c r="A16" s="12" t="s">
+        <v>382</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>304</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>322</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>362</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>323</v>
+      </c>
+      <c r="G16" s="12" t="s">
+        <v>324</v>
+      </c>
+      <c r="H16" s="12" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="46.15" x14ac:dyDescent="0.45">
+      <c r="A17" s="12" t="s">
+        <v>326</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>306</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>307</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>362</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>327</v>
+      </c>
+      <c r="G17" s="12" t="s">
+        <v>328</v>
+      </c>
+      <c r="H17" s="12" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
+      <c r="A18" s="12" t="s">
+        <v>381</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>377</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>376</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>379</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="G18" s="12" t="s">
+        <v>357</v>
+      </c>
+      <c r="H18" s="12" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="E20" s="29"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="B8:C8"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0697A6D-0BB1-44EF-93BC-D89D2D6C44F5}">
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="38.46484375" customWidth="1"/>
+    <col min="2" max="2" width="38.53125" customWidth="1"/>
+    <col min="3" max="3" width="54.265625" customWidth="1"/>
+    <col min="5" max="5" width="46.59765625" customWidth="1"/>
+    <col min="7" max="7" width="40.86328125" customWidth="1"/>
+    <col min="8" max="8" width="68" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="15" x14ac:dyDescent="0.4">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+    </row>
+    <row r="2" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A2" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+    </row>
+    <row r="3" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A3" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>383</v>
+      </c>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+    </row>
+    <row r="5" spans="1:8" ht="15" x14ac:dyDescent="0.4">
+      <c r="A5" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="18"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+    </row>
+    <row r="6" spans="1:8" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A6" s="12" t="s">
+        <v>293</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>294</v>
+      </c>
+      <c r="C6" s="19"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+    </row>
+    <row r="7" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A7" s="12" t="s">
+        <v>295</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>296</v>
+      </c>
+      <c r="C7" s="19"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" s="14"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+    </row>
+    <row r="9" spans="1:8" ht="94.9" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A9" s="27" t="s">
+        <v>359</v>
+      </c>
+      <c r="B9" s="28"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" s="14"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
+    </row>
+    <row r="11" spans="1:8" ht="30" x14ac:dyDescent="0.4">
+      <c r="A11" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="F11" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="G11" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="H11" s="15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="46.15" x14ac:dyDescent="0.45">
+      <c r="A12" s="12" t="s">
+        <v>297</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>293</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>294</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>360</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>298</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
+      <c r="A13" s="12" t="s">
+        <v>300</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>295</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>296</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>360</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="G13" s="12" t="s">
+        <v>301</v>
+      </c>
+      <c r="H13" s="12" t="s">
+        <v>302</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="A9:B9"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: update test case matrix with Menu, Session, and Navigation modules
</commit_message>
<xml_diff>
--- a/test-cases/SauceDemo_TestCases.xlsx
+++ b/test-cases/SauceDemo_TestCases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\saucedemo-playwright-pom\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A25BC20-7664-4CE0-A0D1-CAF6A6DEF68B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EB96396-060E-4603-BE24-9AC4000FC758}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -20,13 +20,16 @@
     <sheet name="Checkout Info" sheetId="5" r:id="rId5"/>
     <sheet name="Checkout Overview" sheetId="6" r:id="rId6"/>
     <sheet name="Checkout Completion" sheetId="7" r:id="rId7"/>
+    <sheet name="Menu" sheetId="8" r:id="rId8"/>
+    <sheet name="Session Management" sheetId="9" r:id="rId9"/>
+    <sheet name="Navigation" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="714" uniqueCount="384">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="891" uniqueCount="470">
   <si>
     <t>Field</t>
   </si>
@@ -1487,6 +1490,499 @@
   </si>
   <si>
     <t>Checkout Completion</t>
+  </si>
+  <si>
+    <t>Menu</t>
+  </si>
+  <si>
+    <t>TS_MENU_001</t>
+  </si>
+  <si>
+    <t>Verify side menu items and their UI behavior</t>
+  </si>
+  <si>
+    <t>TS_MENU_002</t>
+  </si>
+  <si>
+    <t>Verify navigation functionality of side menu items</t>
+  </si>
+  <si>
+    <t>TS_MENU_003</t>
+  </si>
+  <si>
+    <t>Verify Logout functionality</t>
+  </si>
+  <si>
+    <t>TS_MENU_004</t>
+  </si>
+  <si>
+    <t>Verify Reset App State functionality</t>
+  </si>
+  <si>
+    <t>TC_MENU_001</t>
+  </si>
+  <si>
+    <t>Verify all side menu items are visible when menu is opened</t>
+  </si>
+  <si>
+    <t>Common Menu Preconditions</t>
+  </si>
+  <si>
+    <t>Menu items: All Items, About, Logout, Reset App State</t>
+  </si>
+  <si>
+    <t>All four side menu items should be visible.</t>
+  </si>
+  <si>
+    <t>TC_MENU_002</t>
+  </si>
+  <si>
+    <t>Verify side menu item hover changes text color</t>
+  </si>
+  <si>
+    <t>Menu item: About</t>
+  </si>
+  <si>
+    <t>The text color of the About menu item should change to the expected hover color.</t>
+  </si>
+  <si>
+    <t>TC_MENU_003</t>
+  </si>
+  <si>
+    <t>Verify All Items navigation redirects user to Inventory page from Cart page</t>
+  </si>
+  <si>
+    <t>Common Menu Preconditions; 
+User is on the Cart page</t>
+  </si>
+  <si>
+    <t>Menu item: All Items</t>
+  </si>
+  <si>
+    <t>User should be redirected to the Product Inventory page.</t>
+  </si>
+  <si>
+    <t>TC_MENU_004</t>
+  </si>
+  <si>
+    <t>Verify About link redirects user to Sauce Labs external website</t>
+  </si>
+  <si>
+    <t>User should be redirected to the Sauce Labs website.</t>
+  </si>
+  <si>
+    <t>TC_MENU_005</t>
+  </si>
+  <si>
+    <t>Verify Logout redirects user to Login page and clears session</t>
+  </si>
+  <si>
+    <t>Menu item: Logout</t>
+  </si>
+  <si>
+    <t>1. User should be redirected to the Login page. 
+2. Login button should be displayed. 
+3. User session should no longer be active. 
+4. User should not be able to access the Inventory page without logging in.</t>
+  </si>
+  <si>
+    <t>TC_MENU_006</t>
+  </si>
+  <si>
+    <t>Verify Reset App State clears cart items without logging out</t>
+  </si>
+  <si>
+    <t>Common Menu Preconditions; 
+Product is already added to the cart</t>
+  </si>
+  <si>
+    <t>Product: Sauce Labs Fleece Jacket; 
+Menu item: Reset App State</t>
+  </si>
+  <si>
+    <t>1. Cart items should be cleared. 
+2. Cart badge should not be displayed. 
+3. Product should not be present in the cart. 
+4. User should remain logged in.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">Common Menu Preconditions :
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>1. Sauce Demo application is accessible.
+2. User is logged in successfully.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Open the side menu. 
+2. Verify </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>All Items</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> is displayed.
+3. Verify </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">About </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">is displayed.
+4. Verify </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">Logout </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">is displayed.
+5. Verify </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Reset App State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> is displayed.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Open the side menu. 
+2. Hover over the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">About </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>menu item. 
+3. Verify the text color.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Open the side menu. 
+2. Click </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>All Items</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Open the side menu. 
+2. Click </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>About</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Open the side menu. 
+2. Click </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Logout</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>. 
+3. Verify the Login page. 
+4. Verify the login button. 
+5. Attempt to access the Inventory page.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Open the side menu. 
+2. Click </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Reset App State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>. 
+3. Verify the cart badge. 
+4. Open the Cart page. 
+5. Verify the product is no longer in the cart. 
+6. Verify the user remains logged in.</t>
+    </r>
+  </si>
+  <si>
+    <t>TC_MENU_007</t>
+  </si>
+  <si>
+    <t>Verify close menu button closes the side menu</t>
+  </si>
+  <si>
+    <t>Common Menu Preconditions; 
+Menu is open</t>
+  </si>
+  <si>
+    <t>Close menu button</t>
+  </si>
+  <si>
+    <t>1. Open the side menu. 
+2. Verify menu items are visible. 
+3. Click the close menu (X) button. 
+4. Verify menu items are hidden.</t>
+  </si>
+  <si>
+    <t>Side menu should close and menu items should no longer be visible.</t>
+  </si>
+  <si>
+    <t>Session Management</t>
+  </si>
+  <si>
+    <t>TS_SESSION_001</t>
+  </si>
+  <si>
+    <t>TS_SESSION_002</t>
+  </si>
+  <si>
+    <t>Verify unauthenticated access to protected pages is blocked</t>
+  </si>
+  <si>
+    <t>Verify session is fully invalidated after logout</t>
+  </si>
+  <si>
+    <t>TC_SESSION_001</t>
+  </si>
+  <si>
+    <t>TC_SESSION_002</t>
+  </si>
+  <si>
+    <t>TC_SESSION_003</t>
+  </si>
+  <si>
+    <t>TC_SESSION_004</t>
+  </si>
+  <si>
+    <t>TC_SESSION_005</t>
+  </si>
+  <si>
+    <t>Verify direct URL access to Inventory page without login redirects to Login page</t>
+  </si>
+  <si>
+    <t>Verify direct URL access to Cart page without login redirects to Login page</t>
+  </si>
+  <si>
+    <t>Verify direct URL access to Checkout Step One without login redirects to Login page</t>
+  </si>
+  <si>
+    <t>Verify direct URL access to Inventory page after logout redirects to Login page</t>
+  </si>
+  <si>
+    <t>Verify browser back button after logout does not restore authenticated view</t>
+  </si>
+  <si>
+    <t>User logs in then logs out</t>
+  </si>
+  <si>
+    <t>User is not logged in</t>
+  </si>
+  <si>
+    <t>Navigate directly to /inventory.html</t>
+  </si>
+  <si>
+    <t>Navigate directly to /cart.html</t>
+  </si>
+  <si>
+    <t>Navigate directly to /checkout-step-one.html</t>
+  </si>
+  <si>
+    <t>Log out, then navigate directly to /inventory.html</t>
+  </si>
+  <si>
+    <t>Log out, then click browser back button</t>
+  </si>
+  <si>
+    <t>User should be redirected to the Login page</t>
+  </si>
+  <si>
+    <t>Inventory page should not be restored/visible</t>
+  </si>
+  <si>
+    <t>Navigation</t>
+  </si>
+  <si>
+    <t>TC_NAV_001</t>
+  </si>
+  <si>
+    <t>TC_NAV_002</t>
+  </si>
+  <si>
+    <t>TS_NAV_001</t>
+  </si>
+  <si>
+    <t>TS_NAV_002</t>
+  </si>
+  <si>
+    <t>Verify cart badge count persists correctly across navigation</t>
+  </si>
+  <si>
+    <t>User is logged in</t>
+  </si>
+  <si>
+    <t>Navigate directly to /checkout-step-two.html without adding items or completing step one</t>
+  </si>
+  <si>
+    <t>Overview page should show no cart items / no valid order summary</t>
+  </si>
+  <si>
+    <t>Cart badge count should remain accurate (2) throughout navigation</t>
+  </si>
+  <si>
+    <t>Add 2 products from different pages (catalogue + product detail), 
+navigate to cart, then browser-back</t>
+  </si>
+  <si>
+    <t>Verify checkout route access is guarded by completed prior steps</t>
+  </si>
+  <si>
+    <t>Verify cart state remains consistent across page navigation</t>
+  </si>
+  <si>
+    <t>Verify direct URL access to Checkout Step Two without completing 
+Step One does not show valid order data</t>
   </si>
 </sst>
 </file>
@@ -1673,7 +2169,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1712,16 +2208,19 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1735,19 +2234,32 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2037,10 +2549,10 @@
       <c r="A5" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="21"/>
+      <c r="C5" s="22"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
@@ -2051,10 +2563,10 @@
       <c r="A6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="21"/>
+      <c r="C6" s="22"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
@@ -2065,10 +2577,10 @@
       <c r="A7" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="23" t="s">
+      <c r="B7" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="21"/>
+      <c r="C7" s="22"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
@@ -2079,10 +2591,10 @@
       <c r="A8" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="23" t="s">
+      <c r="B8" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="21"/>
+      <c r="C8" s="22"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
@@ -2093,10 +2605,10 @@
       <c r="A9" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="21"/>
+      <c r="C9" s="22"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
@@ -2114,10 +2626,10 @@
       <c r="H10" s="2"/>
     </row>
     <row r="11" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="20" t="s">
+      <c r="A11" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="21"/>
+      <c r="B11" s="22"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
@@ -2136,10 +2648,10 @@
       <c r="H12" s="2"/>
     </row>
     <row r="13" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="20" t="s">
+      <c r="A13" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="21"/>
+      <c r="B13" s="22"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
@@ -2504,6 +3016,163 @@
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B9:C9"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F10BEC3-4884-4769-A8CF-FA1D777F0DBE}">
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="23.59765625" customWidth="1"/>
+    <col min="2" max="2" width="21.19921875" customWidth="1"/>
+    <col min="3" max="3" width="65.06640625" customWidth="1"/>
+    <col min="5" max="5" width="19.59765625" customWidth="1"/>
+    <col min="6" max="6" width="19.06640625" customWidth="1"/>
+    <col min="7" max="7" width="82.796875" customWidth="1"/>
+    <col min="8" max="8" width="57.9296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="15" x14ac:dyDescent="0.4">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A2" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A3" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A4" s="34"/>
+      <c r="B4" s="35"/>
+    </row>
+    <row r="5" spans="1:8" ht="15" x14ac:dyDescent="0.4">
+      <c r="A5" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="17"/>
+    </row>
+    <row r="6" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A6" s="12" t="s">
+        <v>459</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>467</v>
+      </c>
+      <c r="C6" s="18"/>
+    </row>
+    <row r="7" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A7" s="12" t="s">
+        <v>460</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>468</v>
+      </c>
+      <c r="C7" s="18"/>
+    </row>
+    <row r="9" spans="1:8" ht="15" x14ac:dyDescent="0.4">
+      <c r="A9" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="G9" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="H9" s="15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
+      <c r="A10" s="33" t="s">
+        <v>457</v>
+      </c>
+      <c r="B10" s="33" t="s">
+        <v>459</v>
+      </c>
+      <c r="C10" s="30" t="s">
+        <v>469</v>
+      </c>
+      <c r="D10" s="33" t="s">
+        <v>35</v>
+      </c>
+      <c r="E10" s="33" t="s">
+        <v>462</v>
+      </c>
+      <c r="F10" s="33" t="s">
+        <v>91</v>
+      </c>
+      <c r="G10" s="33" t="s">
+        <v>463</v>
+      </c>
+      <c r="H10" s="33" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
+      <c r="A11" s="33" t="s">
+        <v>458</v>
+      </c>
+      <c r="B11" s="33" t="s">
+        <v>460</v>
+      </c>
+      <c r="C11" s="33" t="s">
+        <v>461</v>
+      </c>
+      <c r="D11" s="33" t="s">
+        <v>28</v>
+      </c>
+      <c r="E11" s="33" t="s">
+        <v>462</v>
+      </c>
+      <c r="F11" s="33" t="s">
+        <v>91</v>
+      </c>
+      <c r="G11" s="30" t="s">
+        <v>466</v>
+      </c>
+      <c r="H11" s="33" t="s">
+        <v>465</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2552,97 +3221,97 @@
       <c r="A5" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="25" t="s">
+      <c r="B5" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
     </row>
     <row r="6" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="C6" s="24"/>
-      <c r="D6" s="24"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="25"/>
     </row>
     <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
+      <c r="C7" s="25"/>
+      <c r="D7" s="25"/>
     </row>
     <row r="8" spans="1:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="B8" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="C8" s="24"/>
-      <c r="D8" s="24"/>
+      <c r="C8" s="25"/>
+      <c r="D8" s="25"/>
     </row>
     <row r="9" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
     </row>
     <row r="10" spans="1:8" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="25" t="s">
         <v>81</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="25"/>
     </row>
     <row r="11" spans="1:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="B11" s="24" t="s">
+      <c r="B11" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
+      <c r="C11" s="25"/>
+      <c r="D11" s="25"/>
     </row>
     <row r="12" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="C12" s="24"/>
-      <c r="D12" s="24"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="25"/>
     </row>
     <row r="13" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="B13" s="24" t="s">
+      <c r="B13" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="C13" s="24"/>
-      <c r="D13" s="24"/>
+      <c r="C13" s="25"/>
+      <c r="D13" s="25"/>
     </row>
     <row r="15" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="26" t="s">
         <v>195</v>
       </c>
-      <c r="B15" s="21"/>
+      <c r="B15" s="22"/>
       <c r="C15" s="14"/>
       <c r="D15" s="14"/>
       <c r="E15" s="14"/>
@@ -2661,10 +3330,10 @@
       <c r="H16" s="14"/>
     </row>
     <row r="17" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="27" t="s">
+      <c r="A17" s="19" t="s">
         <v>196</v>
       </c>
-      <c r="B17" s="28"/>
+      <c r="B17" s="20"/>
       <c r="C17" s="14"/>
       <c r="D17" s="14"/>
       <c r="E17" s="14"/>
@@ -3308,17 +3977,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A17:B17"/>
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="B7:D7"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A17:B17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3399,10 +4068,10 @@
       <c r="A5" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="18"/>
+      <c r="C5" s="17"/>
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
       <c r="F5" s="14"/>
@@ -3414,10 +4083,10 @@
       <c r="A6" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>202</v>
       </c>
-      <c r="C6" s="19"/>
+      <c r="C6" s="18"/>
       <c r="D6" s="14"/>
       <c r="E6" s="14"/>
       <c r="F6" s="14"/>
@@ -3429,10 +4098,10 @@
       <c r="A7" s="12" t="s">
         <v>203</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="C7" s="19"/>
+      <c r="C7" s="18"/>
       <c r="D7" s="14"/>
       <c r="E7" s="14"/>
       <c r="F7" s="14"/>
@@ -3444,10 +4113,10 @@
       <c r="A8" s="12" t="s">
         <v>205</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>206</v>
       </c>
-      <c r="C8" s="19"/>
+      <c r="C8" s="18"/>
       <c r="D8" s="14"/>
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
@@ -3478,10 +4147,10 @@
       <c r="I10" s="14"/>
     </row>
     <row r="11" spans="1:9" ht="74.650000000000006" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="27" t="s">
+      <c r="A11" s="19" t="s">
         <v>242</v>
       </c>
-      <c r="B11" s="28"/>
+      <c r="B11" s="20"/>
       <c r="C11" s="14"/>
       <c r="D11" s="14"/>
       <c r="E11" s="14"/>
@@ -3502,10 +4171,10 @@
       <c r="I12" s="14"/>
     </row>
     <row r="13" spans="1:9" ht="70.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="27" t="s">
+      <c r="A13" s="19" t="s">
         <v>243</v>
       </c>
-      <c r="B13" s="28"/>
+      <c r="B13" s="20"/>
       <c r="C13" s="14"/>
       <c r="D13" s="14"/>
       <c r="E13" s="14"/>
@@ -3841,10 +4510,10 @@
       <c r="A5" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="18"/>
+      <c r="C5" s="17"/>
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
       <c r="F5" s="14"/>
@@ -3855,10 +4524,10 @@
       <c r="A6" s="12" t="s">
         <v>245</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>288</v>
       </c>
-      <c r="C6" s="19"/>
+      <c r="C6" s="18"/>
       <c r="D6" s="14"/>
       <c r="E6" s="14"/>
       <c r="F6" s="14"/>
@@ -3869,10 +4538,10 @@
       <c r="A7" s="12" t="s">
         <v>246</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>289</v>
       </c>
-      <c r="C7" s="19"/>
+      <c r="C7" s="18"/>
       <c r="D7" s="14"/>
       <c r="E7" s="14"/>
       <c r="F7" s="14"/>
@@ -3883,10 +4552,10 @@
       <c r="A8" s="12" t="s">
         <v>247</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>290</v>
       </c>
-      <c r="C8" s="19"/>
+      <c r="C8" s="18"/>
       <c r="D8" s="14"/>
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
@@ -3897,10 +4566,10 @@
       <c r="A9" s="12" t="s">
         <v>248</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="18" t="s">
         <v>291</v>
       </c>
-      <c r="C9" s="19"/>
+      <c r="C9" s="18"/>
       <c r="D9" s="14"/>
       <c r="E9" s="14"/>
       <c r="F9" s="14"/>
@@ -3911,10 +4580,10 @@
       <c r="A10" s="12" t="s">
         <v>249</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="18" t="s">
         <v>292</v>
       </c>
-      <c r="C10" s="19"/>
+      <c r="C10" s="18"/>
       <c r="D10" s="14"/>
       <c r="E10" s="14"/>
       <c r="F10" s="14"/>
@@ -3932,10 +4601,10 @@
       <c r="H11" s="14"/>
     </row>
     <row r="12" spans="1:8" ht="97.9" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="16" t="s">
+      <c r="A12" s="28" t="s">
         <v>279</v>
       </c>
-      <c r="B12" s="17"/>
+      <c r="B12" s="29"/>
       <c r="C12" s="14"/>
       <c r="D12" s="14"/>
       <c r="E12" s="14"/>
@@ -4297,10 +4966,10 @@
       <c r="A5" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="18"/>
+      <c r="C5" s="17"/>
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
       <c r="F5" s="14"/>
@@ -4311,10 +4980,10 @@
       <c r="A6" s="12" t="s">
         <v>366</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>330</v>
       </c>
-      <c r="C6" s="19"/>
+      <c r="C6" s="18"/>
       <c r="D6" s="14"/>
       <c r="E6" s="14"/>
       <c r="F6" s="14"/>
@@ -4325,10 +4994,10 @@
       <c r="A7" s="12" t="s">
         <v>367</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>331</v>
       </c>
-      <c r="C7" s="19"/>
+      <c r="C7" s="18"/>
       <c r="D7" s="14"/>
       <c r="E7" s="14"/>
       <c r="F7" s="14"/>
@@ -4339,10 +5008,10 @@
       <c r="A8" s="12" t="s">
         <v>368</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>332</v>
       </c>
-      <c r="C8" s="19"/>
+      <c r="C8" s="18"/>
       <c r="D8" s="14"/>
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
@@ -4360,10 +5029,10 @@
       <c r="H9" s="14"/>
     </row>
     <row r="10" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="27" t="s">
+      <c r="A10" s="19" t="s">
         <v>363</v>
       </c>
-      <c r="B10" s="28"/>
+      <c r="B10" s="20"/>
       <c r="C10" s="14"/>
       <c r="D10" s="14"/>
       <c r="E10" s="14"/>
@@ -4563,7 +5232,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A19" s="12" t="s">
         <v>374</v>
       </c>
@@ -4577,7 +5246,7 @@
         <v>28</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="F19" s="12" t="s">
         <v>91</v>
@@ -4672,10 +5341,10 @@
       <c r="A5" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="18"/>
+      <c r="C5" s="17"/>
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
       <c r="F5" s="14"/>
@@ -4686,10 +5355,10 @@
       <c r="A6" s="12" t="s">
         <v>304</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>305</v>
       </c>
-      <c r="C6" s="19"/>
+      <c r="C6" s="18"/>
       <c r="D6" s="14"/>
       <c r="E6" s="14"/>
       <c r="F6" s="14"/>
@@ -4700,10 +5369,10 @@
       <c r="A7" s="12" t="s">
         <v>306</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>307</v>
       </c>
-      <c r="C7" s="19"/>
+      <c r="C7" s="18"/>
       <c r="D7" s="14"/>
       <c r="E7" s="14"/>
       <c r="F7" s="14"/>
@@ -4714,10 +5383,10 @@
       <c r="A8" s="12" t="s">
         <v>377</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>378</v>
       </c>
-      <c r="C8" s="19"/>
+      <c r="C8" s="18"/>
       <c r="D8" s="14"/>
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
@@ -4735,10 +5404,10 @@
       <c r="H9" s="14"/>
     </row>
     <row r="10" spans="1:8" ht="96.4" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="27" t="s">
+      <c r="A10" s="19" t="s">
         <v>361</v>
       </c>
-      <c r="B10" s="28"/>
+      <c r="B10" s="20"/>
       <c r="C10" s="14"/>
       <c r="D10" s="14"/>
       <c r="E10" s="14"/>
@@ -4939,7 +5608,7 @@
       </c>
     </row>
     <row r="20" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="E20" s="29"/>
+      <c r="E20" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -5023,10 +5692,10 @@
       <c r="A5" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="18"/>
+      <c r="C5" s="17"/>
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
       <c r="F5" s="14"/>
@@ -5037,10 +5706,10 @@
       <c r="A6" s="12" t="s">
         <v>293</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>294</v>
       </c>
-      <c r="C6" s="19"/>
+      <c r="C6" s="18"/>
       <c r="D6" s="14"/>
       <c r="E6" s="14"/>
       <c r="F6" s="14"/>
@@ -5051,10 +5720,10 @@
       <c r="A7" s="12" t="s">
         <v>295</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>296</v>
       </c>
-      <c r="C7" s="19"/>
+      <c r="C7" s="18"/>
       <c r="D7" s="14"/>
       <c r="E7" s="14"/>
       <c r="F7" s="14"/>
@@ -5072,10 +5741,10 @@
       <c r="H8" s="14"/>
     </row>
     <row r="9" spans="1:8" ht="94.9" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A9" s="27" t="s">
+      <c r="A9" s="19" t="s">
         <v>359</v>
       </c>
-      <c r="B9" s="28"/>
+      <c r="B9" s="20"/>
       <c r="C9" s="14"/>
       <c r="D9" s="14"/>
       <c r="E9" s="14"/>
@@ -5180,4 +5849,687 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E46B32F-280A-4BE8-BE02-07D3F3D19A17}">
+  <dimension ref="A1:H20"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.265625" customWidth="1"/>
+    <col min="2" max="2" width="25.6640625" customWidth="1"/>
+    <col min="3" max="3" width="57.6640625" customWidth="1"/>
+    <col min="5" max="5" width="32.06640625" customWidth="1"/>
+    <col min="6" max="6" width="42.796875" customWidth="1"/>
+    <col min="7" max="7" width="51.3984375" customWidth="1"/>
+    <col min="8" max="8" width="49.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="15" x14ac:dyDescent="0.4">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+    </row>
+    <row r="2" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A2" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+    </row>
+    <row r="3" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A3" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>384</v>
+      </c>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+    </row>
+    <row r="5" spans="1:8" ht="15" x14ac:dyDescent="0.4">
+      <c r="A5" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="17"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+    </row>
+    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A6" s="12" t="s">
+        <v>385</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>386</v>
+      </c>
+      <c r="C6" s="18"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+    </row>
+    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="12" t="s">
+        <v>387</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>388</v>
+      </c>
+      <c r="C7" s="18"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+    </row>
+    <row r="8" spans="1:8" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A8" s="12" t="s">
+        <v>389</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>390</v>
+      </c>
+      <c r="C8" s="18"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+    </row>
+    <row r="9" spans="1:8" ht="14.65" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A9" s="12" t="s">
+        <v>391</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>392</v>
+      </c>
+      <c r="C9" s="18"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" s="14"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
+    </row>
+    <row r="11" spans="1:8" ht="60.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A11" s="19" t="s">
+        <v>419</v>
+      </c>
+      <c r="B11" s="20"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
+      <c r="H11" s="14"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" s="14"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="14"/>
+      <c r="G12" s="14"/>
+      <c r="H12" s="14"/>
+    </row>
+    <row r="13" spans="1:8" ht="45" x14ac:dyDescent="0.4">
+      <c r="A13" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="F13" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="G13" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="H13" s="15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A14" s="12" t="s">
+        <v>393</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>385</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>394</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>395</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>396</v>
+      </c>
+      <c r="G14" s="30" t="s">
+        <v>420</v>
+      </c>
+      <c r="H14" s="12" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="46.15" x14ac:dyDescent="0.45">
+      <c r="A15" s="12" t="s">
+        <v>398</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>385</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>399</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>395</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>400</v>
+      </c>
+      <c r="G15" s="30" t="s">
+        <v>421</v>
+      </c>
+      <c r="H15" s="12" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="61.5" x14ac:dyDescent="0.45">
+      <c r="A16" s="12" t="s">
+        <v>402</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>387</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>403</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>404</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>405</v>
+      </c>
+      <c r="G16" s="30" t="s">
+        <v>422</v>
+      </c>
+      <c r="H16" s="12" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="30.75" x14ac:dyDescent="0.45">
+      <c r="A17" s="12" t="s">
+        <v>407</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>387</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>408</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>395</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>400</v>
+      </c>
+      <c r="G17" s="30" t="s">
+        <v>423</v>
+      </c>
+      <c r="H17" s="12" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="76.900000000000006" x14ac:dyDescent="0.45">
+      <c r="A18" s="12" t="s">
+        <v>410</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>389</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>411</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>395</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>412</v>
+      </c>
+      <c r="G18" s="30" t="s">
+        <v>424</v>
+      </c>
+      <c r="H18" s="12" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="92.25" x14ac:dyDescent="0.45">
+      <c r="A19" s="12" t="s">
+        <v>414</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>391</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>415</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>416</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>417</v>
+      </c>
+      <c r="G19" s="30" t="s">
+        <v>425</v>
+      </c>
+      <c r="H19" s="12" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="61.5" x14ac:dyDescent="0.45">
+      <c r="A20" s="12" t="s">
+        <v>426</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>385</v>
+      </c>
+      <c r="C20" s="31" t="s">
+        <v>427</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>428</v>
+      </c>
+      <c r="F20" s="32" t="s">
+        <v>429</v>
+      </c>
+      <c r="G20" s="30" t="s">
+        <v>430</v>
+      </c>
+      <c r="H20" s="31" t="s">
+        <v>431</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="A11:B11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F6E8736-584A-4B14-A289-04D2A34B67BE}">
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.59765625" customWidth="1"/>
+    <col min="2" max="2" width="19.19921875" customWidth="1"/>
+    <col min="3" max="3" width="76.46484375" customWidth="1"/>
+    <col min="5" max="5" width="30.19921875" customWidth="1"/>
+    <col min="6" max="6" width="14.73046875" customWidth="1"/>
+    <col min="7" max="7" width="53.19921875" customWidth="1"/>
+    <col min="8" max="8" width="47.9296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="15" x14ac:dyDescent="0.4">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+    </row>
+    <row r="2" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A2" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+    </row>
+    <row r="3" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A3" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>432</v>
+      </c>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+    </row>
+    <row r="5" spans="1:8" ht="15" x14ac:dyDescent="0.4">
+      <c r="A5" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="17"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+    </row>
+    <row r="6" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A6" s="12" t="s">
+        <v>433</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>435</v>
+      </c>
+      <c r="C6" s="18"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+    </row>
+    <row r="7" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A7" s="12" t="s">
+        <v>434</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>436</v>
+      </c>
+      <c r="C7" s="18"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" s="14"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" s="14"/>
+      <c r="B9" s="14"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+    </row>
+    <row r="10" spans="1:8" ht="15" x14ac:dyDescent="0.4">
+      <c r="A10" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="G10" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="H10" s="15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A11" s="12" t="s">
+        <v>437</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>433</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>442</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>448</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="G11" s="30" t="s">
+        <v>449</v>
+      </c>
+      <c r="H11" s="12" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A12" s="12" t="s">
+        <v>438</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>433</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>443</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>448</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="G12" s="30" t="s">
+        <v>450</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A13" s="12" t="s">
+        <v>439</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>433</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>444</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>448</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="G13" s="30" t="s">
+        <v>451</v>
+      </c>
+      <c r="H13" s="12" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A14" s="12" t="s">
+        <v>440</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>434</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>445</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>447</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="G14" s="30" t="s">
+        <v>452</v>
+      </c>
+      <c r="H14" s="12" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A15" s="12" t="s">
+        <v>441</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>434</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>446</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>447</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="G15" s="30" t="s">
+        <v>453</v>
+      </c>
+      <c r="H15" s="12" t="s">
+        <v>455</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>